<commit_message>
Deploy: 11 May 2026 · COMFORT · add spreadsheet
</commit_message>
<xml_diff>
--- a/Vigil_Content_v2.0.xlsx
+++ b/Vigil_Content_v2.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dominicsmacbook/pCloud Drive/Personal/Vigil/Vigil v2/vigil-build/Vigil/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FC6D94-0B9C-2047-A922-909F590018EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FE3BB9-1C94-D847-9424-9CD0D97FFEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12020" yWindow="660" windowWidth="17320" windowHeight="18460" activeTab="1" xr2:uid="{D95EB6FA-2870-3442-A079-084F9A0CC5D2}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="179">
   <si>
     <t>Hover Links</t>
   </si>
@@ -2580,42 +2580,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Our Lady of Fatima.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Title given to the Virgin Mary following reported apparitions to three shepherd children — Lúcia dos Santos, Francisco Marto and Jacinta Marto — at Fátima, Portugal, between May and October 1917. The Church remembers her today; the memorial falls on this date because 13 May 1917 was the date of the first apparition, and the message carried there was, at its heart, a call to witness and to prayer in a world shaped by conflict.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Author · Acts of the Apostles (1st century AD). </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-Traditionally identified as Luke, a physician and companion of St Paul, and as the author of both the synonymous Gospel and the Acts of the Apostles. He is featured today because Acts 1 gives the disciples — and the reader — their commission: to be witnesses to the risen Christ from Jerusalem to the ends of the earth.</t>
-    </r>
-  </si>
-  <si>
     <t>We are in the fifth week of Eastertide, on the Saturday before the Sixth Sunday of Easter.
 This week, we have moved through love, friendship, choosing, intercession and witness. Saturday in the liturgical week has its own quality — a pause before the Sunday, a moment to let what has been given settle before the arc begins again.</t>
   </si>
@@ -2630,23 +2594,6 @@
     <t>10 May 2026
 6th Sunday of Easter
 Eastertide · Week Six</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">PEACE [pees]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>The English word barely carries what the original means.
-In the Greek of the New Testament, eirēnē (εἰρήνη) translates the Hebrew shalom (שָׁלוֹם) — and shalom is not the absence of conflict. It is a positive condition: wholeness, right relation, the settled flourishing of a life held in proper order before God and neighbour. To greet someone with shalom was not to wish them a quiet life. It was to wish them everything that makes life fully itself.
-When Jesus says "my peace I give to you," he is not offering tranquillity. He is offering participation in the deep order that holds all things — the peace that belongs to someone who knows, even in the darkest hours, that the outcome is not finally in doubt.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -2749,6 +2696,921 @@
         <family val="1"/>
       </rPr>
       <t>Traditionally identified as one of the Twelve Apostles and as the author of the fourth Gospel, three letters and the book of Revelation. He is featured today because John 14 places this gift of peace in the Farewell Discourse — Christ's final private words to his disciples before his death — where it arrives not as reassurance, but as something deliberately left behind.</t>
+    </r>
+  </si>
+  <si>
+    <t>CL-0511</t>
+  </si>
+  <si>
+    <t>11 May 2026
+Monday
+Eastertide · Week Six</t>
+  </si>
+  <si>
+    <t>CL-0512</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">12 May 2026
+Tuesday
+Eastertide · Week Six
+Optional Memorals: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Sts Nereus and Achilleus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, Martyrs
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Pancras</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, Martyr</t>
+    </r>
+  </si>
+  <si>
+    <t>CL-0513</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">13 May 2026
+Tuesday
+Eastertide · Week Six
+Optional Memorals: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Our Lady of Fatima</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Author · Acts of the Apostles (1st century AD). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Traditionally identified as Luke, a physician and companion of St Paul, and as the author of both the synonymous Gospel and the Acts of the Apostles. He is featured today because Acts 1 gives the disciples — and the reader — their commission: to be witnesses to the risen Christ from Jerusalem to the ends of the earth.</t>
+    </r>
+  </si>
+  <si>
+    <t>We are in the sixth week of Eastertide, five weeks on from the resurrection and one week from Pentecost.
+The season is moving toward its close — and as it does, Vigil turns to a word that belongs to this threshold moment: what it means to be held when the one who held you is about to leave.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>"Comfort, O comfort my people,
+says your God.
+Speak tenderly to Jerusalem,
+and cry to her
+that she has served her term,
+that her penalty is paid,
+that she has received from the Lord's hand
+double for all her sins."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Isaiah</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 40:1–2 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You are the God who speaks tenderly — not across the distance, but into it.
+Where grief, fear or weariness has made us feel that you have gone far off, draw near.
+Where we have kept sorrow to ourselves because we were not sure it was permitted, teach us to receive what you are already offering.
+Come close to the places in us that have forgotten how to breathe.
+Let your comfort be not a word spoken at us, but a presence that stays.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Isaiah (8th–6th century BC). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>A prophet of ancient Israel. He wrote at a time when Israel had been conquered by Babylon and its people taken into exile — far from home, far from the Temple, and with the sense that God, who had spoken to and through Israel, had fallen silent because of their disobedience. Isaiah 40 opens with God's first word back into that silence.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Today, when someone offers you kindness — a patient word, an unexpected gesture, a moment of genuine attention — let yourself receive it fully rather than deflecting or minimising it. 
+Do not say it was nothing. Sit with it for a moment and let it be what it is: God speaking tenderly, through an ordinary person, into an ordinary day.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Comfort arrives through hands before it arrives as theology</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">There is a kind of grief that does not want to be argued with. It has heard all the right things said kindly, and it has not moved.
+What it needs is not more words. It needs someone to come in and sit down.
+That is what God commands in Isaiah — not explanation, not theology, but closeness. Speak to the heart. Come in near. The word he uses, nacham, is the word for someone who cannot breathe, being given breath back by another's presence.
+The Spirit Jesus promises is the one who does exactly this — not a message sent from safety, but a presence that comes into the heaviness and stays.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Where has God felt far off to you and why? And is it possible that the distance is not his, but yours?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>We are in the sixth week of Eastertide, moving through the final days before Pentecost.
+Today the Church may remember</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Saints Nereus and Achilleus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Pancras</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> — three early Christians who were put to death for their faith. Their lives ask a question that Eastertide has been building toward: what is it that holds when everything else is taken away?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"Rejoice in the Lord always; again I will say, Rejoice. Let your gentleness be known to everyone. The Lord is near. Do not worry about anything, but in everything by prayer and supplication with thanksgiving let your requests be made known to God. And the peace of God, which surpasses all understanding, will guard your hearts and your minds in Christ Jesus."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Philippians 4:4–7 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Paul writes this from prison. That is not background detail — it is the whole point. He is not describing how he feels. He is describing what he has chosen, and from where.
+Notice what follows immediately after the command to rejoice: do not worry about anything. Paul places them side by side because he knows they cannot both occupy the same ground. Worry insists that the outcome is uncertain and that you are responsible for it. </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Chairō</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> insists that the ground beneath you is held by someone else, regardless of what is happening above it.
+That is not cheerfulness. It is a decision — made before the circumstances change, because it does not depend on them changing.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Where has worry made joy feel not just distant but dishonest? And what would it mean to place that difficulty before God with thanksgiving and to trust that the ground holds?</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You are the ground that holds when everything else feels uncertain.
+Teach us to rejoice not as those who have no difficulties, but as those who know where they stand.
+Where worry has crowded out joy, loosen its grip.
+Where the difficulty is real and the rejoicing feels impossible, meet us there — and let your peace, which we cannot manufacture for ourselves, guard what we cannot protect alone.
+Let what Paul found in a prison cell become real in us today.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Today, when you notice worry beginning to take hold — a problem turned over, a fear rehearsed — stop and name it before God plainly. 
+Then, before you return to it, find one thing in your immediate life to give thanks for. Not to cancel the worry out, but to place both things before God at the same time. 
+That is Paul's move: not pretending the difficulty away, but refusing to let it have the last word.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Rejoicing is not the absence of worry. It is the decision not to let worry pray alone.</t>
+    </r>
+  </si>
+  <si>
+    <t>We are in the sixth week of Eastertide, three days from Pentecost.
+The season is almost complete — and as it closes, Vigil turns to the word that the whole arc of these fifty days has been quietly preparing the reader to receive.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Psalmist</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> does not ask to understand truth, or to be given truth as a possession. The request is simpler and stranger than that: lead me in it. As though truth were a path already laid out ahead — not something the Psalmist constructs by thinking hard enough, but something that requires a guide.
+That is a different relationship to truth than most of us default to. We tend to treat truth as a destination we arrive at through our own effort — research, argument, certainty accumulated over time. The Psalm imagines something less controlling and more trustworthy: truth as the territory God moves through, and the invitation to follow.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>What if the truths you have been trying hardest to work out are less in need of further effort, and more in need of a guide? The Psalmist does not ask to arrive — only to be moving in the right direction, with the right one leading.</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You are the God whose truth holds and whose pathways are laid to guide us.
+Where we have strained after certainty, teach us to be led instead.
+Where we have clutched at answers, open our hands.
+Where we have mistaken our conclusions for your truth, correct us gently.
+Make us to know your ways, and teach us your paths — and let that be enough.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">At some point today, choose one thing you believe to be true — about God, about yourself, about someone you find difficult — and hold it lightly rather than tightly.
+Not to doubt it, but to ask: is this truth? 
+Does it hold because it is real, or because I have needed it to be?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Truth that can bear the weight of that question will still be standing at the end of the day.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Our Lady of Fatima.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Title given to the Virgin Mary following reported apparitions to three shepherd children — Lúcia dos Santos, Francisco Marto and Jacinta Marto — at Fátima, Portugal, between May and October 1917. The Church remembers her today; the memorial falls on this date because 13 May 1917 was the date of the first apparition, and the message carried there was, at its heart, a call to witness and to prayer in a world shaped by conflict.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Author · Psalm 25 (c. 10th century BC). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Traditionally attributed to King David, this is a psalm of petition written in an acrostic form — each verse beginning with a successive letter of the Hebrew alphabet — addressed to God in a time of personal distress and uncertainty. It is featured today because Psalm 25 gives the day's word its deepest register: not truth as argument or possession, but truth as a path into which the Psalmist asks to be led by God.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"Make me to know your ways, O Lord;
+teach me your paths.
+Lead me in your truth, and teach me,
+for you are the God of my salvation;
+for you I wait all day long."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Psalm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 25:4–5 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">TRUTH [trooth]
+The word has been worn smooth by overuse. We reach for it in arguments, to win them. We invoke it to settle things.
+But in the Hebrew of the Old Testament, the word for truth is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>emet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (אֱמֶת) — and </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>emet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> does not primarily mean factual accuracy. It comes from the root aman, meaning to be firm, to hold, to bear weight without giving way. Emet is what does not collapse under you. It is the quality of something you can lean on — not an argument to be won, but a ground to be stood on.
+The Greek word for truth, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>alētheia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (ἀλήθεια), reaches for something slightly different but equally surprising: it means, literally, what is not hidden — what has been brought into the open and can be seen as it actually is.
+Put the two together and you have something worth sitting with. Truth, in scripture, is not something you possess or defeat someone else with. It is something you are led into — a territory more spacious than you expected, and more stable than anything you could have constructed for yourself.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">REJOICE [ri-joiss]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+In ordinary Greek, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>chairō</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (χαίρω) carried the full warmth of the word: celebration, festivity, the mood that belongs to a wedding or a homecoming or good news just arrived. It is the word you use when something has gone well.
+Which is why </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul's</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> use of it is so disorienting. In his letter to the Philippians, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>chairō</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> appears more often than in any other New Testament text — and </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> writes it from prison, to people facing persecution, with the instruction that it applies always. Not when things improve. Not when the fear lifts. Always.
+He says it once, and then — as if he knows the reader will assume he has overstated — he says it again.
+This is not a call to feel cheerful. It is a call to locate your joy somewhere that circumstances cannot reach: in the fact of God, the nearness of Christ, the ground that holds whether the news is good or not. </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> is not asking for something he has never tried. He is asking for it from inside a cell, which is the clearest possible evidence that he believes it can be done.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sts Nereus and Achilleus (1st–2nd century AD).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Early Christian martyrs, traditionally honoured as soldiers in the imperial Roman army who converted to Christianity and refused further military service. The Church remembers them today; their deaths give the day's word its sharpest edge — joy held not as mood but as conviction at the cost of everything.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">St Pancras (c. 289–304 AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">A young Christian martyr, put to death in Rome at approximately fourteen years of age during the persecution under Diocletian. The Church remembers him today; his youth and the sureness of his faith give the day's word a particular force — </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>chairō</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> chosen before a life had fully begun.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">St Paul (1st century AD). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Apostle, missionary and author of letters central to the New Testament. He is featured today because his letter to the Philippians — written from prison — contains the New Testament's most concentrated and insistent use of chairō: rejoice always, and then (in case anyone missed it) rejoice again.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">COMFORT [kum-fert]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+The word has grown soft in ordinary use. We reach for it when someone is sad and we want to say something kind. But comfort, in its full biblical register, is not softness at all.
+The Hebrew word at the heart of </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Isaiah</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 40 is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>nacham</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (נָחַם) — to breathe again, to be brought back to breath. It is the word for someone crushed under a weight so heavy they can no longer draw air, and then relieved of it. 
+When the Jewish scholars who translated the Old Testament into Greek rendered this word, they chose </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>parakaleō</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (παρακαλέω): to call someone to your side, to come in close, to strengthen from within. It is the root of the word </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>paraklētos</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> — the name Jesus gives the Holy Spirit that he will send after he is gone.
+Comfort, then, is not a gentle word spoken from across the room. It is the movement of God into the place where someone cannot breathe.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">PEACE [pees]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">The English word barely carries what the original means.
+In the Greek of the New Testament, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>eirēnē</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (εἰρήνη) translates the Hebrew </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>shalom</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (שָׁלוֹם) — and shalom is not the absence of conflict. It is a positive condition: wholeness, right relation, the settled flourishing of a life held in proper order before God and neighbour. To greet someone with shalom was not to wish them a quiet life. It was to wish them everything that makes life fully itself.
+When Jesus says "my peace I give to you," he is not offering tranquillity. He is offering participation in the deep order that holds all things — the peace that belongs to someone who knows, even in the darkest hours, that the outcome is not finally in doubt.</t>
     </r>
   </si>
 </sst>
@@ -3004,7 +3866,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -3112,6 +3974,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="2" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3650,7 +4515,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="10"/>
@@ -3917,7 +4782,7 @@
         <v>130</v>
       </c>
       <c r="I9" s="28" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -3928,7 +4793,7 @@
         <v>133</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D10" s="25" t="s">
         <v>134</v>
@@ -3949,34 +4814,165 @@
         <v>139</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="405" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="C11" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="D11" s="25" t="s">
+        <v>178</v>
+      </c>
+      <c r="E11" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="C11" s="24" t="s">
-        <v>144</v>
-      </c>
-      <c r="D11" s="25" t="s">
+      <c r="F11" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="G11" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="F11" s="24" t="s">
+      <c r="H11" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="I11" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="H11" s="24" t="s">
+    </row>
+    <row r="12" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="I11" s="28" t="s">
+      <c r="B12" s="37" t="s">
         <v>151</v>
       </c>
+      <c r="C12" s="24" t="s">
+        <v>157</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>177</v>
+      </c>
+      <c r="E12" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="F12" s="24" t="s">
+        <v>162</v>
+      </c>
+      <c r="G12" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="I12" s="28" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>175</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="F13" s="24" t="s">
+        <v>165</v>
+      </c>
+      <c r="G13" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="I13" s="28" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="F14" s="24" t="s">
+        <v>169</v>
+      </c>
+      <c r="G14" s="27" t="s">
+        <v>170</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="I14" s="28" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="22"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="28"/>
+    </row>
+    <row r="16" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="22"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="28"/>
+    </row>
+    <row r="17" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="28"/>
+    </row>
+    <row r="18" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="22"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
Fix notification delivery — midnight UTC send_after, 7:45 AM delivery
</commit_message>
<xml_diff>
--- a/Vigil_Content_v2.0.xlsx
+++ b/Vigil_Content_v2.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dominicsmacbook/pCloud Drive/Personal/Vigil/Vigil v2/vigil-build/Vigil/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2FE3BB9-1C94-D847-9424-9CD0D97FFEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61972F28-3AE9-B346-90A2-1703A6A2CFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12020" yWindow="660" windowWidth="17320" windowHeight="18460" activeTab="1" xr2:uid="{D95EB6FA-2870-3442-A079-084F9A0CC5D2}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29340" windowHeight="18460" activeTab="1" xr2:uid="{D95EB6FA-2870-3442-A079-084F9A0CC5D2}"/>
   </bookViews>
   <sheets>
     <sheet name="April" sheetId="3" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="233">
   <si>
     <t>Hover Links</t>
   </si>
@@ -2758,24 +2758,6 @@
   </si>
   <si>
     <t>CL-0513</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">13 May 2026
-Tuesday
-Eastertide · Week Six
-Optional Memorals: </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>Our Lady of Fatima</t>
-    </r>
   </si>
   <si>
     <r>
@@ -3613,12 +3595,1544 @@
 When Jesus says "my peace I give to you," he is not offering tranquillity. He is offering participation in the deep order that holds all things — the peace that belongs to someone who knows, even in the darkest hours, that the outcome is not finally in doubt.</t>
     </r>
   </si>
+  <si>
+    <t>CL-0514</t>
+  </si>
+  <si>
+    <t>CL-0515</t>
+  </si>
+  <si>
+    <t>CL-0516</t>
+  </si>
+  <si>
+    <t>14 May 2026
+Thursday
+Eastertide · Week Six
+Solemnity · The Ascension of the Lord</t>
+  </si>
+  <si>
+    <t>We are in Eastertide, and today the Church keeps the Solemnity of the Ascension — the fortieth day of the great fifty, when the risen Christ is taken up in glory and the disciples are left standing, looking upward, between what has been and what is coming.
+This is not an ending. It is the hinge on which everything turns.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>ASCEND [uh-SEND]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+To ascend is not to disappear. It is to enter more fully into the place from which all things are governed.
+The Greek word used in Acts is analēmpsis (ἀνάλημψις) — a taking up, a receiving into — and what is received is not a ghost or a spirit, but a body: the same body that was broken and raised, now carried into the presence of God. 
+In the Psalms, ascent language belongs to worship — the pilgrim going up to Jerusalem, moving toward the place where heaven and earth meet. 
+The Ascension of Christ does not abolish that language. It fulfils it: the one who goes up is not leaving the world behind, but drawing it after him into God.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>"God put this power to work in Christ when he raised him from the dead and seated him at his right hand in the heavenly places, far above all rule and authority and power and dominion, and above every name that is named, not only in this age but also in the age to come."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Ephesians 1:20–21 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Paul (1st century AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Apostle, missionary and author of letters central to the New Testament. He is featured today because the Letter to the Ephesians gives the Ascension its most precise theological framing: not absence, but enthronement — Christ raised and seated above every power that claims authority over the world.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">There is a temptation, on the Ascension, to read it as loss — the one who was near becoming remote, the visible becoming invisible. The disciples standing on the hillside feel it. They are left looking at the sky.
+But </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul's</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> language in Ephesians does not describe distance. It describes authority: Christ seated at God's right hand, far above every power that competes for the governance of the world. The Ascension is not Christ retreating from history. It is Christ enthroned over it.
+That distinction matters for the ordinary life of faith. The one you pray to is not absent and sympathetic. He is present and sovereign — which is a different kind of comfort, and a more demanding one.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Where have you been treating Christ as someone who has gone away and left you to manage, rather than as the one in whose hands everything already rests? If Christ is not absent but enthroned — governing, not withdrawn — what would you do differently today with that knowledge fully in view?</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You ascended not to leave us, but to reign over every power, every fear, every thing that seems to be in charge of our lives.
+Where we have behaved as though the world were unguided, remind us that you holds it in your arms.
+Where we have mistaken your hiddenness for absence, open our eyes.
+Let the same power that raised you from the dead be at work in us. Make us less afraid of what is coming, because we know where you are seated.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Choose one responsibility or anxiety you have been treating as the load you alone must carry. Not to put it down — it may be real and serious — but to carry it differently.
+Before you return to it today, look up — physically, deliberately — and name it before God. Say: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>I am not above this. But you are.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Then return to it — not as the person responsible for the outcome, but as someone working under a governance that holds even this.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>That is what it means to live after the Ascension.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">15 May 2026
+Friday
+Eastertide ·  Week Six
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Isidore the Farmer</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">We are in the sixth week of Eastertide, the day after the Ascension — the season in its final stretch with Pentecost just one week away.
+Today the Church may remember </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Isidore the Farmer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, a labourer whose ordinary life became, across its length, an act of prayer.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">TEND [tend]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+To tend is not to control. It is to give consistent, unglamorous attention to something that cannot grow by force.
+The Hebrew </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>shamar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (שָׁמַר) — to keep, to watch over, to guard — runs through the creation narratives and the psalms as the word for what is entrusted to human care.
+In Genesis, the human creature is placed in the garden not to possess it but to till and to keep it: to bring faithful attention to bear on something whose life is given, not made. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Isidore</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> spent his working life doing precisely that, in a single field, over many years. He did not change the world. He tended it.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Isidore the Farmer (c. 1070–1130 AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Spanish agricultural labourer, canonised in 1622, patron saint of farmers and of Madrid. The Church remembers him today; his life gives the day's word its most concrete instance — faithfulness not as achievement but as daily, unglamorous tending of what has been given.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Author · Psalm 121 (c. 10th–6th century BC). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">One of the Songs of Ascent — psalms sung by pilgrims travelling up to Jerusalem for the great feasts. It is featured today because Psalm 121 gives the word </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>shamar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> its fullest devotional range: the God who tends his people with an attention that never fails.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"The Lord is your keeper;
+the Lord is your shade at your right hand.
+The sun shall not strike you by day,
+nor the moon by night.
+The Lord will keep you from all evil;
+he will keep your life.
+The Lord will keep
+your going out and your coming in
+from this time on and for evermore."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Psalm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 121:5–8 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The same word — </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>shamar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, to tend or keep — belongs both to the human creature in the garden and to God watching over the pilgrim on the road. 
+That is not coincidence. It is the shape of the whole relationship: we are called to tend what we have been given because we ourselves are tended by one whose attention does not waver.
+Most of what we tend never makes news. A friendship kept alive by small regular acts of faithfulness. A habit of prayer returned to on the days when it costs something. A piece of work done carefully when no one is watching.
+St Isidore's life was not dramatic. But the tradition has remembered it for nine centuries, which is its own kind of testimony about what faithfulness looks like when you stay with it.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Some things in your life are tended; others are merely handled. The difference is not the size of the thing or the time you give it, but whether you are truly present to it. What is asking for your presence — not your efficiency — today?</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You are the keeper who does not sleep, present at our going out and our coming in.
+Teach us to tend what you have given us — not to impress, not to achieve, but because faithful attention is the shape love takes over time.
+Where we have neglected the small things in hope of larger ones, call us back.
+Where we have become weary of the unremarkable, let us find you there.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">At some point today, do one ordinary thing — make a drink, walk a familiar route, return a message you have been putting off — and do it slowly, as an act of deliberate attention rather than efficient completion.
+Before you begin, name it before God: this is what I am tending. I offer you my attention to it.
+The word </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>shamar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> does not mean doing more. It means being present to what you are already doing, as though it were worth your full care.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Tending is not a task to complete. It is a posture to practise.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">16 May 2026
+Saturday
+Eastertide · Week Six
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Simon Stock</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">We are in the sixth week of Eastertide, on the Saturday before Pentecost — the last full day of the great fifty, one threshold away from the coming of the Spirit.
+The Church may remember today </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Simon Stock</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, who lived most of his life in waiting, and whose patience became a kind of prophecy.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>WAIT [wayt]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+To wait is not to be passive. It is to hold yourself in readiness for something you cannot produce.
+The Hebrew </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qavah</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (קָוָה) — to wait, but also to hope, to stretch toward — carries a quality of active tension rather than passive endurance. The root image is of a cord drawn taut: something under pressure, straining in one direction, held firm by the expectation of what is coming. 
+In the Psalms, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qavah</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> is the posture of the soul before God on the edge of dawn, through the darkest hours, believing that morning is coming before the sky shows any sign of it.</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You ask us to wait — not as those who have been forgotten, but as those who know what is coming.
+Where our restlessness has mistaken activity for faithfulness, help us to be still.
+Where we have grown impatient with your timing, teach us the posture of those who watch for the morning.
+Hold us in readiness for what only you can give.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">At some point today, when you feel the pull to check, to plan, to move on to the next thing — pause instead. Physically stop. Let thirty seconds become a minute.
+In that pause, name before God one thing you have been trying to force into resolution. Do not pray for a solution. Simply hold it open, as a question rather than a problem, and say: I am waiting for you in this.
+The Psalmist who watched for the morning did not make the sun rise. He simply remained awake and oriented until it did.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>That is the whole practice: to remain awake, and to stay facing the right direction.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Simon Stock (c. 1165–1265 AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">English friar and prior general of the Carmelites, an order of religious life rooted in a tradition of solitary prayer and watchful waiting. The Church remembers him today; his life of contemplative perseverance gives the day's word its particular depth.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Author · Psalm 130 (c. 10th–6th century BC). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>One of the seven Penitential Psalms and one of the Songs of Ascent — a psalm of waiting from within distress. It is featured today because Psalm 130 gives qavah its most concentrated expression: not passive endurance, but active, tensed hope held through the dark.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"I wait for the Lord, my soul waits,
+and in his word I hope;
+my soul waits for the Lord
+more than those who watch for the morning,
+more than those who watch for the morning."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Psalm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 130:5–6 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Psalmist</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> repeats the image — more than those who watch for the morning, more than those who watch for the morning — because saying it once is not enough. This is not a quick glance toward the horizon. It is a long watching, a posture held through the night.
+The disciples, in the days between the Ascension and the coming of the Spirit at Pentecost, are told to wait — not to go back to their old lives, not to manufacture what they need, but to remain and receive what is promised. 
+That waiting is not wasted time. It is the necessary form of a trust that cannot be forced.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Waiting feels unproductive because we measure time by what we make of it. But qavah — the stretched, taut waiting of the Psalmist — is not empty. It is oriented. Where are you being asked to stop producing and start receiving, and what would it cost you to trust that the waiting itself is the right response?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">13 May 2026
+Wednesday
+Eastertide · Week Six
+Optional Memorals: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Our Lady of Fatima</t>
+    </r>
+  </si>
+  <si>
+    <t>CL-0517</t>
+  </si>
+  <si>
+    <t>CL-0518</t>
+  </si>
+  <si>
+    <t>CL-0519</t>
+  </si>
+  <si>
+    <t>17 May 2026
+7th Sunday of Easter
+Eastertide · Week Seven</t>
+  </si>
+  <si>
+    <t>We are in Eastertide, on the Seventh Sunday of Easter — one week from Pentecost, the last Sunday of the great fifty days.
+Today, Vigil turns to a word that belongs to this threshold: a word that sounds like it refers to something distant and overwhelming, but turns out to describe something much closer to home.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"O Lord, our Sovereign, how majestic is your name in all the earth!
+When I look at your heavens, the work of your fingers,
+the moon and the stars that you have established;
+what are human beings that you are mindful of them,
+mortals that you care for them?
+Yet you have made them a little lower than God,
+and crowned them with glory and honour."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Psalm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 8:1, 3–5 (NRSV)</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You made us to carry something of your weight in the world — and we have mostly forgotten this.
+Where we have made ourselves smaller than you made us, remind us.
+Where we have treated our own lives as unimportant, or the lives of others as disposable, correct us.
+Restore in us the dignity of people who bear your image — not as pride, but as responsibility.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Identify the one voice — a memory, a comparison, a habit of self-description — that most consistently persuades you that your life does not weigh very much.
+Every time you hear it today, answer it with the plain fact: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>"I was made in the image of someone whose name is majestic in all the earth."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 
+That is not arrogance. It is accuracy.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Glory was not something you had to earn. It was given. The practice is learning to stop arguing with the gift.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Author · Psalm 8 (c. 10th century BC).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Traditionally attributed to King David, this is a psalm of praise addressed to God as Creator. It is featured today because it contains one of scripture's most surprising claims: that </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>kabod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> — the word for God's own weight and glory — belongs also to human beings, given by God before any achievement or merit.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>GLORY [GLAW-ree]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+In Hebrew, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>kabod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (כָּבוֹד) comes from a root meaning weight — heaviness, substance, the quality of something that cannot be ignored or passed through. The </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>kabod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> of God is not brightness as decoration. It is the felt reality of a presence too substantial for the world around it to simply absorb.
+When the writers of the Old Testament use </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>kabod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> of human beings — and they do — something unexpected happens. A person of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>kabod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> is not famous or impressive. They are real in a way that commands attention. The honour given to a parent, the weight a judge carries, the dignity of a life faithfully lived: these are </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>kabod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> too. 
+The word does not belong only to the heavens. It belongs wherever something is genuinely what it is.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Psalmist</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> starts where most of us start: with the sky, and the sudden sense of smallness. The moon and the stars that you established. Beside all that, what are we?
+The expected answer is: not much. The actual answer is stranger than that.
+You have crowned them with glory and honour. The same word — </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>kabod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> — that belongs to the presence of God is given here to human beings. Not because they have earned it, but because this is what it means to be human: to carry something of that weight in the world.
+Most of us do not feel glorious. We feel tired, partial, smaller than we hoped. And yet the Psalmist will not let that feeling be the last word.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>When did you last feel the full weight of your own life — not your achievements or your failures, but simply the fact of being someone God made and has not stopped being mindful of? And what has been quietly convincing you, since then, that it was a mistake rather than the truest thing about you?</t>
+    </r>
+  </si>
+  <si>
+    <t>18 May 2026
+Monday
+Eastertide · Week Seven</t>
+  </si>
+  <si>
+    <t>We are in the seventh and final week of Eastertide, two days from Pentecost.
+The great fifty days are almost over. This week Vigil turns to a word that belongs to the threshold: what it means to come through something without being undone by it.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">OVERCOME [oh-ver-KUM]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+The Greek word is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>nikaō</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (νικάω) — to conquer, to prevail, to pass through something and emerge on the other side still yourself. In the ancient world it belonged to the language of battle and contest: Nike, the goddess of victory, gave the word its most familiar face.
+But in the New Testament, nikaō migrates somewhere quieter. It describes not the person who was protected from difficulty, but the person who went through it and was not finally destroyed by it. The one who nikaō does not avoid the fight. They come out the other side.
+There is a compound form — </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>hypernikaō</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> — that intensifies this further. Not merely to overcome, but to overcome beyond overcoming: to come through so completely that even the struggle has been made to serve something.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>"Who will separate us from the love of Christ? Will hardship, or distress, or persecution, or famine, or nakedness, or peril, or sword? No, in all these things we are more than conquerors through him who loved us."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Romans</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 8:35, 37 (NRSV)</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You know what we are carrying — the hardship that is real, the fear that has made itself at home, the thing we have let write our conclusions for too long.
+We are not asking you to remove it. We are asking you to be more present in it than it is.
+Let the love that neither hardship nor peril can separate us from be more solid, today, than the weight of what presses against us.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">There is something in your life — you know what it is — that has been acting as though it has the final word. And there is almost certainly someone in your life carrying the same weight: the person who has gone quiet, the friend whose difficulty you have been meaning to acknowledge, the one for whom the hardship or distress or loss is very present today.
+Contact them. Not to fix anything. Not with a solution or a verse or an encouragement. Simply to say: I have been thinking of you, and I am not going anywhere.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>That is what it looks like to be, for one person, the evidence that love cannot be separated from them by what they are going through. Hypernikaō, enacted in an ordinary day.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Paul (1st century AD).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Apostle and author of letters central to the New Testament. He wrote the Letter to the Romans to a community facing a real danger of torture or execution for their faith, so when he lists hardships, he is not speaking in abstractions. He is featured today because Romans 8 gives the day's word its most searching expression: not that suffering is avoided, but that it cannot separate those who are loved by God from that love.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The word overcome doesn't appear in that passage. What appears instead is "more than conquerors" — and in the Greek, that is a single word: hypernikaō. The word we began with, pressed to its furthest point.
+In writing the Letter to the Romans, </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> does not say the hardships listed go away. He names them plainly — hardship, distress, famine, peril, sword — because he is writing to people living under Roman rule, many of them from the poorest classes in society or even slaves, and many facing real danger for their faith. 
+So he is not offering comfort to people who might one day suffer. He is writing to people already in it, and saying: even so, none of this separates you from the love of God.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul's point is not that suffering must be extreme to count. It is that nothing — of any size, any kind — falls outside the reach of this love. What have you been carrying without bringing it to God, not because it felt too heavy, but because you were not sure it was worth his attention?</t>
+    </r>
+  </si>
+  <si>
+    <t>We are in Eastertide, on the eve of Pentecost — the last day of the great fifty, the threshold before the Spirit comes.
+Tomorrow the season ends and a new one begins. Today is a day for standing still before what is about to arrive.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">HOLY [HOH-lee]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+The Hebrew root is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qadosh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (קָדוֹשׁ) — set apart, cut off from the ordinary, other than what surrounds it. In the Hebrew scriptures, the word first belongs to God alone: the sound of the one thing in existence that is wholly what it is, uncorrupted and unlike anything else.
+But </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qadosh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> does not stay with God. It moves. The altar is holy because it is where God is approached. The day is holy because it is set aside for God. And in the New Testament, the people of God are holy — not because they have achieved moral perfection, but because they have been set apart: drawn into relation with the one who is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qadosh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> in himself, and beginning, slowly, to be changed by that proximity.
+The Greek word for holy, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>hagios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (ἅγιος), carries the same weight. The Holy Spirit is not only a spirit that is morally good. It is the Spirit who is other — who brings the presence of the utterly different into the ordinary life of the world. 
+And tomorrow, on Pentecost, that Spirit arrives.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"I saw the Lord sitting on a throne, high and lofty; and the hem of his robe filled the temple. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Seraphs</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> were in attendance above him; each had six wings: with two they covered their faces, and with two they covered their feet, and with two they flew. 
+And one called to another and said: 'Holy, holy, holy is the Lord of hosts; the whole earth is full of his glory.'"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Isaiah</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 6:1b–3 (NRSV)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Isaiah (8th–7th century BC).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">A prophet of ancient Israel, writing at a time of political turmoil and moral crisis among God's people. He is featured today because the vision recorded at the opening of his prophetic calling — in which he sees God enthroned and the whole earth declared full of divine glory — gives the day's word its deepest register: holiness not as moral tidiness but as the overwhelming reality of God's presence breaking into ordinary life.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Seraphs.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Heavenly figures described in the vision of the prophet Isaiah as attendants around the throne of God. The Hebrew word saraph means burning one. They are depicted with six wings — two covering their faces before the divine presence, two covering their feet in reverence, and two for flight. They appear in this passage and nowhere else in the Hebrew scriptures.</t>
+    </r>
+  </si>
+  <si>
+    <t>19 May 2026
+Tuesday
+Eastertide · Week Seven
+Eve of Pentecost</t>
+  </si>
+  <si>
+    <t>Lord,
+You are holy — utterly unlike anything else, and yet present in the ordinary rooms and ordinary days of ordinary people.
+Tomorrow your Spirit arrives. Today we bring you what we are: distracted, incomplete, not as ready as we would like to be.
+We are not asking to be overwhelmed. We are asking to be open.
+Come, Holy Spirit, into the ordinary ground of this life. Find whatever room there is, and fill it.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Before the day is over, do one thing to make yourself genuinely available to what is coming — not by becoming more impressive or more prepared, but by removing something that has been filling the space.
+Identify one thing that has been occupying the room: a distraction returned to too often, a resentment kept close, a busyness that has crowded out quiet. Set it down deliberately before God today — not permanently, not with great drama, but as a single act of making space.
+The Holy Spirit does not wait for perfect conditions. But </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Isaiah</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> was in the temple. The disciples were gathered and waiting. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Availability is not the same as worthiness. It is simply the decision to be present to what is already here.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Isaiah went to the temple to pray. He was not looking for what happened. And yet the utterly different — the one the seraphs cannot look at directly — filled the room he was standing in.
+That is what </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qadosh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> does. It does not wait for the right conditions or the right person. It breaks through into ordinary life because ordinary life is already full of it, whether the people inside it know it or not.
+Tomorrow, on Pentecost, the Holy Spirit came upon the followers of Jesus — not in a grand public place but in a room, among ordinary people who did not fully know what they were waiting for.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>You are reading this in your own ordinary place, on the day before. Isaiah was not prepared. The disciples had been told to wait but did not know for what. Neither preparedness nor understanding was the condition. What would it mean, today, to simply make yourself present — and willing to be surprised?</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3674,6 +5188,20 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FF3D4A5C"/>
+      <name val="Georgia"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -3987,8 +5515,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF3D4A5C"/>
       <color rgb="FFFFFDF5"/>
-      <color rgb="FF3D4A5C"/>
       <color rgb="FFF2EBE0"/>
       <color rgb="FF8C8680"/>
       <color rgb="FFFFFFFF"/>
@@ -4515,7 +6043,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="10"/>
@@ -4782,7 +6310,7 @@
         <v>130</v>
       </c>
       <c r="I9" s="28" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -4825,7 +6353,7 @@
         <v>143</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>145</v>
@@ -4851,25 +6379,25 @@
         <v>151</v>
       </c>
       <c r="C12" s="24" t="s">
+        <v>156</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="E12" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="D12" s="24" t="s">
-        <v>177</v>
-      </c>
-      <c r="E12" s="26" t="s">
+      <c r="F12" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="G12" s="27" t="s">
         <v>158</v>
       </c>
-      <c r="F12" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="G12" s="27" t="s">
+      <c r="H12" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="I12" s="28" t="s">
         <v>159</v>
-      </c>
-      <c r="H12" s="24" t="s">
-        <v>161</v>
-      </c>
-      <c r="I12" s="28" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -4880,25 +6408,25 @@
         <v>153</v>
       </c>
       <c r="C13" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="E13" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="F13" s="24" t="s">
+        <v>164</v>
+      </c>
+      <c r="G13" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="I13" s="28" t="s">
         <v>175</v>
-      </c>
-      <c r="E13" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="F13" s="24" t="s">
-        <v>165</v>
-      </c>
-      <c r="G13" s="27" t="s">
-        <v>166</v>
-      </c>
-      <c r="H13" s="24" t="s">
-        <v>167</v>
-      </c>
-      <c r="I13" s="28" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -4906,75 +6434,217 @@
         <v>154</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>155</v>
+        <v>205</v>
       </c>
       <c r="C14" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>173</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="F14" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="D14" s="24" t="s">
-        <v>174</v>
-      </c>
-      <c r="E14" s="26" t="s">
-        <v>173</v>
-      </c>
-      <c r="F14" s="24" t="s">
+      <c r="G14" s="27" t="s">
         <v>169</v>
       </c>
-      <c r="G14" s="27" t="s">
+      <c r="H14" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="H14" s="24" t="s">
+      <c r="I14" s="28" t="s">
         <v>171</v>
       </c>
-      <c r="I14" s="28" t="s">
-        <v>172</v>
-      </c>
     </row>
-    <row r="15" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="22"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="28"/>
+    <row r="15" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>181</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="E15" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="F15" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="G15" s="27" t="s">
+        <v>187</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="I15" s="28" t="s">
+        <v>185</v>
+      </c>
     </row>
-    <row r="16" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="22"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="28"/>
+    <row r="16" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>191</v>
+      </c>
+      <c r="E16" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="F16" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="G16" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>196</v>
+      </c>
+      <c r="I16" s="28" t="s">
+        <v>192</v>
+      </c>
     </row>
-    <row r="17" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="22"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="26"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="28"/>
+    <row r="17" spans="1:9" ht="374" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>198</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>199</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>203</v>
+      </c>
+      <c r="F17" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="G17" s="27" t="s">
+        <v>200</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="I17" s="28" t="s">
+        <v>202</v>
+      </c>
     </row>
-    <row r="18" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="22"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="28"/>
+    <row r="18" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>210</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>215</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>211</v>
+      </c>
+      <c r="F18" s="24" t="s">
+        <v>216</v>
+      </c>
+      <c r="G18" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="H18" s="24" t="s">
+        <v>213</v>
+      </c>
+      <c r="I18" s="28" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="22" t="s">
+        <v>207</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>217</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>218</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>219</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="G19" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>222</v>
+      </c>
+      <c r="I19" s="28" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="22" t="s">
+        <v>208</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>229</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>225</v>
+      </c>
+      <c r="D20" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="E20" s="24" t="s">
+        <v>227</v>
+      </c>
+      <c r="F20" s="24" t="s">
+        <v>232</v>
+      </c>
+      <c r="G20" s="27" t="s">
+        <v>230</v>
+      </c>
+      <c r="H20" s="24" t="s">
+        <v>231</v>
+      </c>
+      <c r="I20" s="28" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="22"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="28"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="30" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Deploy: 23 May 2026 · OPEN · cache vigil-v63
</commit_message>
<xml_diff>
--- a/Vigil_Content_v2.0.xlsx
+++ b/Vigil_Content_v2.0.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dominicsmacbook/pCloud Drive/Personal/Vigil/Vigil v2/vigil-build/Vigil/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61972F28-3AE9-B346-90A2-1703A6A2CFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6055D966-6C87-9143-96B1-BD63771C0194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29340" windowHeight="18460" activeTab="1" xr2:uid="{D95EB6FA-2870-3442-A079-084F9A0CC5D2}"/>
+    <workbookView xWindow="12000" yWindow="660" windowWidth="17400" windowHeight="18460" activeTab="1" xr2:uid="{D95EB6FA-2870-3442-A079-084F9A0CC5D2}"/>
   </bookViews>
   <sheets>
     <sheet name="April" sheetId="3" r:id="rId1"/>
     <sheet name="May" sheetId="2" r:id="rId2"/>
+    <sheet name="June" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">April!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">June!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">May!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="336">
   <si>
     <t>Hover Links</t>
   </si>
@@ -3173,72 +3175,6 @@
         <family val="1"/>
       </rPr>
       <t xml:space="preserve"> 25:4–5 — NRSV</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">TRUTH [trooth]
-The word has been worn smooth by overuse. We reach for it in arguments, to win them. We invoke it to settle things.
-But in the Hebrew of the Old Testament, the word for truth is </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>emet</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (אֱמֶת) — and </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>emet</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> does not primarily mean factual accuracy. It comes from the root aman, meaning to be firm, to hold, to bear weight without giving way. Emet is what does not collapse under you. It is the quality of something you can lean on — not an argument to be won, but a ground to be stood on.
-The Greek word for truth, </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>alētheia</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (ἀλήθεια), reaches for something slightly different but equally surprising: it means, literally, what is not hidden — what has been brought into the open and can be seen as it actually is.
-Put the two together and you have something worth sitting with. Truth, in scripture, is not something you possess or defeat someone else with. It is something you are led into — a territory more spacious than you expected, and more stable than anything you could have constructed for yourself.</t>
     </r>
   </si>
   <si>
@@ -4186,43 +4122,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">St Simon Stock (c. 1165–1265 AD). 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">English friar and prior general of the Carmelites, an order of religious life rooted in a tradition of solitary prayer and watchful waiting. The Church remembers him today; his life of contemplative perseverance gives the day's word its particular depth.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-Author · Psalm 130 (c. 10th–6th century BC). 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>One of the seven Penitential Psalms and one of the Songs of Ascent — a psalm of waiting from within distress. It is featured today because Psalm 130 gives qavah its most concentrated expression: not passive endurance, but active, tensed hope held through the dark.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <rPr>
         <i/>
         <sz val="12"/>
@@ -4435,40 +4334,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Author · Psalm 8 (c. 10th century BC).
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">Traditionally attributed to King David, this is a psalm of praise addressed to God as Creator. It is featured today because it contains one of scripture's most surprising claims: that </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>kabod</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> — the word for God's own weight and glory — belongs also to human beings, given by God before any achievement or merit.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <rPr>
         <b/>
         <sz val="12"/>
@@ -4647,10 +4512,6 @@
     <t>18 May 2026
 Monday
 Eastertide · Week Seven</t>
-  </si>
-  <si>
-    <t>We are in the seventh and final week of Eastertide, two days from Pentecost.
-The great fifty days are almost over. This week Vigil turns to a word that belongs to the threshold: what it means to come through something without being undone by it.</t>
   </si>
   <si>
     <r>
@@ -4833,112 +4694,6 @@
     </r>
   </si>
   <si>
-    <t>We are in Eastertide, on the eve of Pentecost — the last day of the great fifty, the threshold before the Spirit comes.
-Tomorrow the season ends and a new one begins. Today is a day for standing still before what is about to arrive.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">HOLY [HOH-lee]
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">
-The Hebrew root is </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>qadosh</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (קָדוֹשׁ) — set apart, cut off from the ordinary, other than what surrounds it. In the Hebrew scriptures, the word first belongs to God alone: the sound of the one thing in existence that is wholly what it is, uncorrupted and unlike anything else.
-But </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>qadosh</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> does not stay with God. It moves. The altar is holy because it is where God is approached. The day is holy because it is set aside for God. And in the New Testament, the people of God are holy — not because they have achieved moral perfection, but because they have been set apart: drawn into relation with the one who is </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>qadosh</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> in himself, and beginning, slowly, to be changed by that proximity.
-The Greek word for holy, </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>hagios</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (ἅγιος), carries the same weight. The Holy Spirit is not only a spirit that is morally good. It is the Spirit who is other — who brings the presence of the utterly different into the ordinary life of the world. 
-And tomorrow, on Pentecost, that Spirit arrives.</t>
-    </r>
-  </si>
-  <si>
     <r>
       <rPr>
         <i/>
@@ -5038,12 +4793,6 @@
       </rPr>
       <t>Heavenly figures described in the vision of the prophet Isaiah as attendants around the throne of God. The Hebrew word saraph means burning one. They are depicted with six wings — two covering their faces before the divine presence, two covering their feet in reverence, and two for flight. They appear in this passage and nowhere else in the Hebrew scriptures.</t>
     </r>
-  </si>
-  <si>
-    <t>19 May 2026
-Tuesday
-Eastertide · Week Seven
-Eve of Pentecost</t>
   </si>
   <si>
     <t>Lord,
@@ -5092,7 +4841,282 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Isaiah went to the temple to pray. He was not looking for what happened. And yet the utterly different — the one the seraphs cannot look at directly — filled the room he was standing in.
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>TRUTH [trooth]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+The word has been worn smooth by overuse. We reach for it in arguments, to win them. We invoke it to settle things.
+But in the Hebrew of the Old Testament, the word for truth is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>emet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (אֱמֶת) — and </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>emet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> does not primarily mean factual accuracy. It comes from the root aman, meaning to be firm, to hold, to bear weight without giving way. Emet is what does not collapse under you. It is the quality of something you can lean on — not an argument to be won, but a ground to be stood on.
+The Greek word for truth, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>alētheia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (ἀλήθεια), reaches for something slightly different but equally surprising: it means, literally, what is not hidden — what has been brought into the open and can be seen as it actually is.
+Put the two together and you have something worth sitting with. Truth, in scripture, is not something you possess or defeat someone else with. It is something you are led into — a territory more spacious than you expected, and more stable than anything you could have constructed for yourself.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Psalmist · Psalm 8 (c. 10th century BC).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Traditionally attributed to King David, this is a psalm of praise addressed to God as Creator. It is featured today because it contains one of scripture's most surprising claims: that </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>kabod</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> — the word for God's own weight and glory — belongs also to human beings, given by God before any achievement or merit.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Simon Stock (c. 1165–1265 AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">English friar and prior general of the Carmelites, an order of religious life rooted in a tradition of solitary prayer and watchful waiting. The Church remembers him today; his life of contemplative perseverance gives the day's word its particular depth.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Psalmist · Psalm 130 (c. 10th–6th century BC).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>The Psalms were composed by many hands across the centuries and the identity of most authors is unknown.  Psalm 130 is one of the Penitential Psalms and the Songs of Ascent. It is featured today because it gives qavah its most concentrated expression: not passive endurance, but active, tensed hope held through the dark.</t>
+    </r>
+  </si>
+  <si>
+    <t>We are in the seventh and final week of Eastertide, with less than a week until Pentecost.
+The great fifty days are almost over. This week Vigil turns to a word that belongs to the threshold: what it means to come through something without being undone by it.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">HOLY [HOH-lee]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+The Hebrew root is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qadosh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (קָדוֹשׁ) and means that which is set apart, cut off from the ordinary, other than what surrounds it.  In the Hebrew scriptures, the word first belongs to God alone: the sound of the one thing in existence that is wholly what it is, uncorrupted and unlike anything else.
+But </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qadosh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> does not stay with God. It moves. The altar is holy because it is where God is approached. The day is holy because it is set aside for God. And in the New Testament, the people of God are holy — not because they have achieved moral perfection, but because they have been set apart: drawn into relation with the one who is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>qadosh</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> in himself, and beginning, slowly, to be changed by that proximity.
+The Greek word for holy, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>hagios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (ἅγιος), carries the same weight. The Holy Spirit is not only a spirit that is morally good. It is the Spirit who is other — who brings the presence of the utterly different into the ordinary life of the world. 
+And tomorrow, on Pentecost, that Spirit arrives.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Isaiah</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> went to the temple to pray. He was not looking for what happened. And yet the utterly different — the one the seraphs cannot look at directly — filled the room he was standing in.
 That is what </t>
     </r>
     <r>
@@ -5125,6 +5149,1688 @@
         <family val="1"/>
       </rPr>
       <t>You are reading this in your own ordinary place, on the day before. Isaiah was not prepared. The disciples had been told to wait but did not know for what. Neither preparedness nor understanding was the condition. What would it mean, today, to simply make yourself present — and willing to be surprised?</t>
+    </r>
+  </si>
+  <si>
+    <t>CL-0520</t>
+  </si>
+  <si>
+    <t>19 May 2026
+Tuesday
+Eastertide · Week Seven</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">20 May 2026
+Wednesday
+Eastertide · Week Seven
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Bernadine of Siena</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, priest</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>"Therefore God also highly exalted him and gave him the name that is above every name, so that at the name of Jesus every knee should bend, in heaven and on earth and under the earth, and every tongue should confess that Jesus Christ is Lord, to the glory of God the Father."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Philippians 2:9–11 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">NAME [naym]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+In the ancient Greco-Roman world, a name was not simply a label. 
+Onoma (ὄνομα) — the Greek word </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> uses in his letter to the Philippians — carried the person's identity, authority and honour within it. To act in someone's name was to act with their full weight behind you. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> knew this, and he also knew something older behind it. In the Hebrew scriptures, shem (שֵׁם) — the word for name — carried the same concentrated sense. This is why the divine name is treated so carefully throughout scripture — not as a magic word, but as the concentrated reality of who God is. 
+When </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> writes of a name above every name, he is drawing on both registers at once: the Greek world his Philippian readers inhabited, and the Jewish inheritance that shaped everything he knew about God.
+The name above every name, in that light, is not a label promoted above others. It is the one name that carries the full weight of who Christ is — and what that weight can bear.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Most of us have inherited the name of Jesus as a given — something received so early and repeated so often that for many, it passes through the mouth without always passing through the mind.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul's</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> letter to the Philippians pushes back against that. The name he is writing about is not a formula. It carries the full weight of who Christ is — the presence, the authority and the capacity to act. A name, in the world Paul inhabited, was not a label attached from outside. It was the thing itself.
+A thousand years after </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Bernardine of Siena</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> spent thirty years travelling the length of Italy on foot, drawing crowds of thousands in town squares, and directing everything — every sermon, every journey — toward a single point: the name of Jesus as the centre of Christian life. Not a system. Not a theology to be mastered. A name to be returned to.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Where in your life has the name of Jesus become background noise? When did you last say it slowly, meaning it? And what do you find, or fail to find, when you bring it into the room with whatever you are carrying today?</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You gave to Christ the name that is above every name — and you gave it as a gift, not a title.
+Where we have said your name without thinking, teach us to say it again.
+Where your name has become familiar in the wrong way — worn smooth by habit, emptied by repetition — restore its weight.
+Let what we say with our mouths become what we carry in our lives.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">At some point today, say the name of Jesus — not in a prayer, not in a formula, but deliberately, as an act of attention. Say it once and hold it for a moment, as though you were handing something solid rather than sounding a noise.
+Bernardine believed that a name held up in silence could do more than an hour of eloquent speech. He may have been right.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>The name is not a password. It is a presence.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Bernardine of Siena (1380–1444 AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Italian priest and member of the Franciscans — a Christian religious order committed to poverty, preaching and travelling ministry.  His entire ministry was built on the theology of the Holy Name of Jesus, which he promoted through the IHS monogram — the first three letters of Jesus' name in Greek — becoming the most celebrated itinerant preacher of fifteenth-century Italy.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">St Paul (1st century AD). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Apostle, missionary and author of letters central to the New Testament. He is featured today because the Christ-hymn in Philippians 2 gives the day's word its fullest register: the name above every name is not a title awarded to Jesus but the concentrated substance of who he is, given by God in response to a life of complete self-emptying.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">We are in the seventh and final week of Eastertide, four days from Pentecost. 
+The great fifty days are almost complete, and as they close, many Christian traditions remember </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Bernardine of Siena</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> — a Franciscan friar whose life was given, from beginning to end, to a single word: the name of Jesus.</t>
+    </r>
+  </si>
+  <si>
+    <t>CL-0521</t>
+  </si>
+  <si>
+    <t>CL-0522</t>
+  </si>
+  <si>
+    <t>CL-0523</t>
+  </si>
+  <si>
+    <t>CL-0524</t>
+  </si>
+  <si>
+    <t>CL-0525</t>
+  </si>
+  <si>
+    <t>CL-0526</t>
+  </si>
+  <si>
+    <t>CL-0527</t>
+  </si>
+  <si>
+    <t>CL-0528</t>
+  </si>
+  <si>
+    <t>CL-0529</t>
+  </si>
+  <si>
+    <t>CL-0530</t>
+  </si>
+  <si>
+    <t>CL-0531</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">21 May 2026
+Thursday
+Eastertide · Week Seven
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Christopher Magallanes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, priest, and companions, martyrs</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">22 May 2026
+Friday
+Eastertide · Week Seven
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Rita of Cassia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, religious</t>
+    </r>
+  </si>
+  <si>
+    <t>23 May 2026
+Saturday
+Eastertide · Week Seven</t>
+  </si>
+  <si>
+    <t>28 May 2026
+Thursday
+Ordinary Time · Week One</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">27 May 2026
+Wednesday
+Ordinary Time · Week One
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Augustine of Canterbury</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, bishop</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">29 May 2026
+Friday
+Ordinary Time · Week One
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Paul VI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, pope</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">25 May 2026
+Monday
+Ordinary Time · Week One
+Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>The Blessed Virgin Mary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, Mother of the Church</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">30 May 2026
+Saturday
+Ordinary Time · Week One
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>The Blesssed Virgin Mary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> on Saturday</t>
+    </r>
+  </si>
+  <si>
+    <t>31 May 2026
+Sunday
+Ordinary Time · Week Two
+Solemnity: The Most Holy Trinity</t>
+  </si>
+  <si>
+    <t>24 May 2026
+Sunday
+Eastertide · Week Seven
+Solemnity: Pentecost</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">26 May 2026
+Tuesday
+Ordinary Time · Week One
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Philip Neri</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, priest</t>
+    </r>
+  </si>
+  <si>
+    <t>CH-0601</t>
+  </si>
+  <si>
+    <t>CH-0602</t>
+  </si>
+  <si>
+    <t>CH-0603</t>
+  </si>
+  <si>
+    <t>CH-0604</t>
+  </si>
+  <si>
+    <t>CH-0605</t>
+  </si>
+  <si>
+    <t>CH-0606</t>
+  </si>
+  <si>
+    <t>CH-0607</t>
+  </si>
+  <si>
+    <t>CH-0608</t>
+  </si>
+  <si>
+    <t>CH-0609</t>
+  </si>
+  <si>
+    <t>CH-0610</t>
+  </si>
+  <si>
+    <t>CH-0611</t>
+  </si>
+  <si>
+    <t>CH-0612</t>
+  </si>
+  <si>
+    <t>CH-0613</t>
+  </si>
+  <si>
+    <t>CH-0614</t>
+  </si>
+  <si>
+    <t>CH-0615</t>
+  </si>
+  <si>
+    <t>CH-0616</t>
+  </si>
+  <si>
+    <t>CH-0617</t>
+  </si>
+  <si>
+    <t>CH-0618</t>
+  </si>
+  <si>
+    <t>CH-0619</t>
+  </si>
+  <si>
+    <t>CH-0620</t>
+  </si>
+  <si>
+    <t>CH-0621</t>
+  </si>
+  <si>
+    <t>CH-0622</t>
+  </si>
+  <si>
+    <t>CH-0623</t>
+  </si>
+  <si>
+    <t>CH-0624</t>
+  </si>
+  <si>
+    <t>CH-0625</t>
+  </si>
+  <si>
+    <t>CH-0626</t>
+  </si>
+  <si>
+    <t>CH-0627</t>
+  </si>
+  <si>
+    <t>CH-0628</t>
+  </si>
+  <si>
+    <t>CH-0629</t>
+  </si>
+  <si>
+    <t>CH-0630</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">02 June 2026
+Tuesday
+Ordinary Time · Week Two
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Marcellinus and St Peter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, martyrs</t>
+    </r>
+  </si>
+  <si>
+    <t>04 June 2026
+Thursday
+Ordinary Time · Week Two</t>
+  </si>
+  <si>
+    <t>07 June 2026
+Sunday
+Ordinary Time · Week Three
+Solemnity: The Most Sacred Heart of Jesus</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">03 June 2026
+Wednesday
+Ordinary Time · Week Two
+Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Charles Lwanga and companions</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, martyrs</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">05 June 2026
+Friday
+Ordinary Time · Week Two
+Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Boniface</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, bishop and martyr</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">06 June 2026
+Saturday
+Ordinary Time · Week Two
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Norbert</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, bishop
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>The Blessed Virgin Mary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> on Saturday</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">01 June 2026
+Monday
+Ordinary Time · Week Two
+Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Justin Martyr</t>
+    </r>
+  </si>
+  <si>
+    <t>We are in Eastertide, on the eve of Pentecost — the last few days of the great fifty, the threshold before the Spirit comes.
+Very soon, the season ends and a new one begins. Today is a day for standing still before what is about to arrive.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Forgiveness is easy to praise and difficult to practise, because practising it requires acknowledging that something real was done — that the wound was not imaginary and the wrong not minor. The temptation is to short-circuit this by moving quickly to the language of forgiveness without passing through the fact of injury.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul's</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> instruction in Colossians does not bypass the wound. It acknowledges a complaint — a real grievance between real people — and then asks something costly: to respond to it in the way God has responded to you.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Christopher Magallanes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> was arrested on false charges, given no trial and executed. His last recorded words were not a claim to justice, but an absolution: "I am innocent and die innocent. I absolve with all my heart those who seek my death and ask God that my blood bring peace to a divided Mexico." He did not pretend the wrong was not real. He released the claim anyway.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Where have you been holding a complaint that has not yet become forgiveness — and what do you imagine it would cost you to let it go?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Christopher Magallanes (1869–1927).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Mexican diocesan priest. The Church remembers him today with his twenty-four companions — priests and laymen killed during the Cristero War, a period of violent anti-Catholic persecution in Mexico. He was arrested while travelling to celebrate Mass on a farm, given no trial and executed. His last words were an act of forgiveness and a prayer for peace.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+St Paul (1st century AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Apostle, missionary and author of letters central to the New Testament. He is featured today because his letter to the Colossians gives the day's word its most searching instruction: to forgive one another as the Lord has forgiven us — not as a counsel of naïve optimism, but as a response to a grace already received.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">We are in the seventh and final week of Eastertide, three days before Pentecost.
+Today the Church remembers </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Christopher Magallanes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> and twenty-four companions, priests and laypeople who were killed in Mexico in the 1920s and who went to their deaths with forgiveness on their lips.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">FORGIVE [fer-GIV]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+To forgive is not to pretend that the wrong did not happen. 
+It is to release the claim it has on you and to release your claim against the person who inflicted it.
+The Greek aphiēmi (ἀφίημι) means to send away, to let go, to release. In the New Testament it is used both for the forgiveness of sins and for the release of debts.
+The two meanings are not coincidental: the debt language speaks to a God who is owed something and chooses to cancel it; the sin language speaks to a God whose standard has been violated and who chooses not to prosecute — in both cases, the initiative of forgiveness is entirely God's.</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You have forgiven more in us than we know how to name — without waiting for us to deserve it.
+Where we are carrying wounds we have not yet named to you, give us the honesty to speak them.
+Where we have been wronged, help us to let the forgiveness you have shown us become the forgiveness we offer in turn
+Give us the courage to release what we have been carrying, and the grace to carry it no longer.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">At some point today, write down — briefly, honestly — one grievance you have been holding: what was done, and by whom. Let the writing be as plain as possible, without drama.
+Then set the pen down, and say once: I forgive this. Not because the wrong was small, but because you are no longer willing to carry it. If the feeling does not follow immediately, that is normal. The act precedes the feeling.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>The forgiveness that changes us usually begins before we feel ready to give it.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">We are in the seventh and final week of Eastertide, two days from Pentecost.
+Today the Church remembers </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Rita of Cascia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> — a fifteenth-century nun whose long life became, in ways she could not have planned, an answer to a single question: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>what does it mean to follow?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>FOLLOW [FOL-oh]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+To follow is to move in someone else's direction, at their pace, toward a destination they have chosen rather than you.
+The Greek </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>akolouthein</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (ἀκολουθεῖν) is used throughout the New Testament almost exclusively for discipleship. It is not the word for walking behind someone in a crowd. It is the word for a deliberate reorientation of a life — giving up the right to set your own course and moving instead in the direction of another.
+What makes the word unusual is what it does not require. It does not require understanding the destination. It does not require feeling ready. In almost every instance where Jesus uses it in the Gospels, the person called to follow has no map, no guarantee and no particular preparation. They are simply asked whether they will go.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>"Bear with one another and, if anyone has a complaint against another, forgive each other; just as the Lord has forgiven you, so you also must forgive."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Colossians 3:13 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You call us to follow you — not in the abstract, but from the actual circumstances of our lives.
+Where we have been dragging our feet, give us the grace to move.
+When we are afraid of where you are leading us, meet us with your presence.
+Teach us to trust that you know the road, even when we cannot see it.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Rita of Cascia (1381–1457). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Italian Augustinian nun. She is associated with impossible causes and with a life shaped, at every stage, by unchosen suffering which she came to embrace as a form of following Christ into his Passion. She bore a wound on her forehead — understood as a partial stigmata from Christ's Crown of Thorns — for the last fifteen years of her life.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+St Peter (1st century AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Traditionally identified as one of the Twelve Apostles, a leading witness to the resurrection and as the author of two letters in the New Testament. He is featured today because the First Letter of Peter addresses communities facing persecution and suffering, and gives the day's word its clearest theological grounding: the call to follow Christ is not a call away from difficulty but into it, in His steps.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Identify one person in your life in whom you can see something of Christ — a patience, a steadiness, a quality of faith you recognise as real. 
+Reach out to them today in some form: a message, a call, a question. Let their direction become, for a moment, your direction.
+And if you find the openness to go further, you might ask them how they have learned to follow — what it has cost them, and what it has given them.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>We often learn to follow Christ by first learning to follow those in whom his life is visible.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Following, as the New Testament means it, is not the same as agreeing with someone's ideas. It requires a genuine reorientation — turning toward God, and moving in that direction even when the path is not the one you would have chosen.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Rita of Cascia</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> wanted to give her life to God in one way. God led her through another: marriage, widowhood, years of refusal before she finally entered the convent. At each stage she had to choose, again, whether to follow God within the life she actually had — not the life she had planned.
+Rita's life was not what she expected. But at each stage, God was present in it — and accessible to her precisely because she stopped fighting the shape of it and began following within it.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Where in your own life have you been waiting for better conditions before you follow — before you pray, before you trust, before you give God the part of your life you have been holding back? What would it mean to follow from exactly where you are now?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"For to this you have been called, because Christ also suffered for you, leaving you an example, so that you should follow in his steps."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+1 </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Peter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 2:21 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <t>We are at the end of the great fifty days. Eastertide closes today — one day before Pentecost, when the Church waits for what Christ promised before he left.
+The waiting is almost over.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Being open is harder than it sounds, because most of us are only selectively open — ready to receive the things we were already hoping for, and guarded against the rest.
+The disciples waiting before Pentecost had no clear picture of what was coming. They had been told to wait, and that something would arrive — but the shape of it was unknown. What the Spirit required of them before it came was not understanding, not preparation, and not worthiness. It required only that they stay in the room.
+There are parts of your life where you have been expecting God to act — and where, over time, the expectation may have hardened into a particular shape: the specific outcome, the particular answer, the change that would look exactly the way you imagined. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Where might that expectation itself be the obstruction — and what would it mean, today, to release the shape of what you are waiting for, and simply remain open?</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You promised to send what your people needed, and you kept that promise.
+Where we have been waiting with clenched hands, open them.
+Where we have decided the shape of what you will give, help us to let that go.
+Where fear has made us guarded, make us available.
+We do not know what you are about to do. We are asking only to be open when you do it.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Before the day ends, choose one area of your life where you have been waiting for God to act — and where, honestly, you have already decided what the answer should look like.
+Hold that expectation for a moment. Then, deliberately, loosen your grip on it. Not in resignation, but in trust: the one who is coming knows better than you do what you need.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Openness is not passivity. It is the active decision to stop obstructing what God wants to give.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Paul (1st century AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Apostle, missionary and author of letters central to the New Testament. He is featured today because the final verses of the Acts of the Apostles show him in Rome — under arrest, under guard — proclaiming the Kingdom of God with complete freedom and without hindrance. It is from his situation that the day's word takes its deepest meaning.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>OPEN [OH-pen]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+To be open is not simply to be unlocked. It is to be without obstruction — available, undefended, ready to receive what comes.
+The Greek </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>akōlytōs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (ἀκωλύτως) means unhindered, unimpeded, free from obstacle. In the final lines of the Acts of the Apostles, it is the word used to describe how </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> proclaimed the Kingdom of God in Rome for two years — not freely in the sense of being unguarded, but freely in the sense of being unblocked, the message moving without restraint from a man under house arrest.
+There is something striking in that. The obstruction was still there — the chains, the soldier, the appeal to Caesar — and yet the word that closes the whole account of the early Church is this one: unhindered. What was open was not the door, but the proclamation that went through it.
+On the last day before Pentecost, the question the word puts to the reader is not whether the way ahead is clear. It is whether you are open to what God is about to do.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">"He lived there for two full years at his own expense and welcomed all who came to him, proclaiming the kingdom of God and teaching about the Lord Jesus Christ with all boldness and without hindrance."
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Acts 28:30–31 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <t>Eastertide ends today. 
+The great fifty days — which began at Easter and have carried the Church through resurrection, ascension and expectation — reach their completion in the feast of Pentecost.
+This is the day the Spirit came.</t>
+  </si>
+  <si>
+    <t>Lord,
+You did not leave your people to manage alone. You promised the Spirit, and you sent the Spirit, and the Spirit has not been withdrawn.
+Where we have been trying to live the Christian life on our own resources, remind us what you gave us.
+Where we have grown tired, breathe.
+Where we have grown cold, kindle.
+Where we have grown silent, speak through us in ways we could not have found ourselves.
+Come, Holy Spirit.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">What arrived at Pentecost did not arrive quietly. It arrived as wind and fire — disruptive, unmistakable, impossible to ignore. The disciples in that room had been waiting, praying and keeping still. They had done everything that could be done from the human side.
+And then something happened that they could not have produced by their own waiting.
+That is the character of the Spirit throughout scripture: it is not generated, it is received. It comes from outside the system. It does not reward effort in the way that effort normally expects to be rewarded. It comes when and how it will — which is not an argument against preparation, but an argument against the assumption that preparation is what causes the arrival.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Where in your life have you been trying to generate what can only be received — working to produce a quality of faith, peace or love that is, in the end, a gift? 
+And what would it mean to stop producing and simply become the kind of person through whom the Spirit can move?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>SPIRIT [SPIR-it]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+In the original languages of scripture, the word for spirit carries more than one meaning at once — and that is not an accident.
+The Hebrew </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>ruach</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (רוּחַ) means wind, breath and spirit. The Greek </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>pneuma</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (πνεῦμα) carries the same range. In both cases, what the word holds together is the movement of an invisible force that is known not by being seen but by what it does: the breath that animates a body, the wind that bends the trees, the spirit that moves through and beyond what is merely physical.
+This is why, when the Spirit arrives at Pentecost, it arrives as wind and fire — not as metaphors added afterward to explain something, but as the thing itself in its most recognisable forms. The word was never only spiritual in the modern, ethereal sense. It was always also breath. Always also force.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>"When the day of Pentecost had come, they were all together in one place. 
+And suddenly from heaven there came a sound like the rush of a violent wind, and it filled the entire house where they were sitting. 
+Divided tongues, as of fire, appeared among them, and a tongue rested on each of them. 
+All of them were filled with the Holy Spirit and began to speak in other languages, as the Spirit gave them ability."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Acts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 2:1–4 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Choose one thing today that you have been trying to do in your own strength — a conversation you have been dreading, a habit you have been fighting, a relationship you have been managing — and before you face it, pause and ask the Spirit to go with you into it.
+Not a long prayer. A single breath, and the simplest of requests:
+Come, Holy Spirit.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Veni, Sancte Spiritus.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>The Spirit does not need elaborate invitation. It needs only the door to be open.</t>
+    </r>
+  </si>
+  <si>
+    <t>We are at the start of Ordinary Time — the first Monday after Pentecost, and the first weekday of a new season.
+Ordinary Time is not a diminishment. It is the season in which what was given at Easter and Pentecost is carried into the whole ordinary length of a life. 
+The Church begins it today by remembering Mary — present at the Annunciation, present at the cross, and present in the Upper Room when the Spirit came. She is the one figure who stands at every threshold of the story, and the Church calls her its mother.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">MOTHERHOOD [MU-thər-hud]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+The word comes from the Old English modor — one who carries, tends and forms — and it has always meant more than biological origin. A mother is the one in whose care something comes to be itself.
+The Church's claim that Mary is its mother rests on a specific observation: she was there. At the Annunciation, she received the Word before anyone else. And in the days between the Ascension and Pentecost, she was in the Upper Room with the apostles, praying with them as they waited for the Spirit who would bring the Church to life.
+Acts places her there in a single, quiet phrase — Mary the mother of Jesus — among the disciples, at prayer, before everything began. She is not leading. She is not speaking. She is present, and she is praying. 
+The Church has understood that as a form of motherhood: not the motherhood of authority, but of faithful, sustaining presence at the moment of birth.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>"All these were constantly devoting themselves to prayer, together with certain women, including Mary the mother of Jesus, as well as his brothers."</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Acts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 1:14 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Mary carried Christ — literally, bodily — and then spent the rest of her life releasing him: to his ministry, to the disciples, to the cross, to the Church.
+Motherhood, in her case, was inseparable from the willingness to let go of what she had carried.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>What are you holding onto that belongs, now, in someone else's hands? Identify it. Then find one concrete act today that begins the transfer.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The description in Acts is almost aggressively ordinary. 
+Mary, identified only by her relationship to Jesus, is doing what everyone else is doing. But she had already lived through the Annunciation, the cross, and everything in-between, and she knew something about carrying that the others were only beginning to learn.
+That is what Luke's account of her shows, from beginning to end: a life shaped by receiving something not asked for, carrying it at cost, and releasing it when the time came. 
+At the Annunciation she received. At the cross she held on. In the Upper Room she let the Church be born from what she had carried.
+Motherhood, in this sense, is not possession. It is the willingness to carry something fully and then to release it into the world rather than keep it for yourself.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>What have you been carrying — a person, a responsibility, a vision for someone else's life — that may now be asking to be released rather than held?</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You gave your Church a mother who knew how to carry and how to release.
+Where we have confused holding on with faithfulness, show us the difference.
+Where we have carried something that was never ours to keep — a person, a hope, a vision for someone else's life — give us the courage to open our hands.
+Let what we have carried with love be released with love, as she did.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Author · Acts of the Apostles (1st century AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFF0E0D0"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Traditionally identified as Luke, a physician and companion of St Paul, and as the author of both the synonymous Gospel and the Acts of the Apostles. He is featured today because the opening of Acts 2 is his account of the Spirit's arrival at Pentecost — the event that closes Eastertide and opens the life of the Church.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Author · Acts of the Apostles (1st century AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Traditionally identified as Luke, a physician and companion of St Paul, and as the author of both the synonymous Gospel and the Acts of the Apostles. He is featured today because it is in Acts 1 that Mary appears for the last time in the New Testament, as the Church waits for the Spirit that will bring it to life.</t>
     </r>
   </si>
 </sst>
@@ -5132,7 +6838,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5203,8 +6909,42 @@
       <name val="Georgia"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFF0E0D0"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FFF0E0D0"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFF0E0D0"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color rgb="FFF0E0D0"/>
+      <name val="Georgia"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFF0E0D0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5244,6 +6984,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFDF5"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC04040"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC04040"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -5394,7 +7146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -5507,6 +7259,27 @@
     <xf numFmtId="15" fontId="2" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5515,6 +7288,8 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFF0E0D0"/>
+      <color rgb="FFC04040"/>
       <color rgb="FF3D4A5C"/>
       <color rgb="FFFFFDF5"/>
       <color rgb="FFF2EBE0"/>
@@ -6043,7 +7818,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="10"/>
@@ -6353,7 +8128,7 @@
         <v>143</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>145</v>
@@ -6382,7 +8157,7 @@
         <v>156</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E12" s="26" t="s">
         <v>157</v>
@@ -6411,7 +8186,7 @@
         <v>162</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E13" s="26" t="s">
         <v>163</v>
@@ -6426,7 +8201,7 @@
         <v>166</v>
       </c>
       <c r="I13" s="28" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -6434,13 +8209,13 @@
         <v>154</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>167</v>
       </c>
       <c r="D14" s="24" t="s">
-        <v>173</v>
+        <v>225</v>
       </c>
       <c r="E14" s="26" t="s">
         <v>172</v>
@@ -6460,180 +8235,757 @@
     </row>
     <row r="15" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="22" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B15" s="37" t="s">
+        <v>180</v>
+      </c>
+      <c r="C15" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="D15" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="E15" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="F15" s="24" t="s">
+        <v>185</v>
+      </c>
+      <c r="G15" s="27" t="s">
+        <v>186</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="I15" s="28" t="s">
         <v>184</v>
-      </c>
-      <c r="F15" s="24" t="s">
-        <v>186</v>
-      </c>
-      <c r="G15" s="27" t="s">
-        <v>187</v>
-      </c>
-      <c r="H15" s="24" t="s">
-        <v>188</v>
-      </c>
-      <c r="I15" s="28" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="22" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B16" s="37" t="s">
+        <v>188</v>
+      </c>
+      <c r="C16" s="24" t="s">
         <v>189</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="D16" s="24" t="s">
         <v>190</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="E16" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="F16" s="24" t="s">
+        <v>193</v>
+      </c>
+      <c r="G16" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="H16" s="24" t="s">
+        <v>195</v>
+      </c>
+      <c r="I16" s="28" t="s">
         <v>191</v>
-      </c>
-      <c r="E16" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="F16" s="24" t="s">
-        <v>194</v>
-      </c>
-      <c r="G16" s="27" t="s">
-        <v>195</v>
-      </c>
-      <c r="H16" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="I16" s="28" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="374" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="22" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B17" s="37" t="s">
+        <v>196</v>
+      </c>
+      <c r="C17" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="D17" s="24" t="s">
         <v>198</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="E17" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="F17" s="24" t="s">
+        <v>202</v>
+      </c>
+      <c r="G17" s="27" t="s">
         <v>199</v>
       </c>
-      <c r="E17" s="24" t="s">
-        <v>203</v>
-      </c>
-      <c r="F17" s="24" t="s">
+      <c r="H17" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="I17" s="28" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="G17" s="27" t="s">
-        <v>200</v>
-      </c>
-      <c r="H17" s="24" t="s">
-        <v>201</v>
-      </c>
-      <c r="I17" s="28" t="s">
-        <v>202</v>
+      <c r="B18" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>208</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>212</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="F18" s="24" t="s">
+        <v>213</v>
+      </c>
+      <c r="G18" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="H18" s="24" t="s">
+        <v>211</v>
+      </c>
+      <c r="I18" s="28" t="s">
+        <v>226</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
-        <v>206</v>
-      </c>
-      <c r="B18" s="23" t="s">
-        <v>209</v>
-      </c>
-      <c r="C18" s="24" t="s">
-        <v>210</v>
-      </c>
-      <c r="D18" s="24" t="s">
+    <row r="19" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="22" t="s">
+        <v>205</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>214</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>228</v>
+      </c>
+      <c r="D19" s="24" t="s">
         <v>215</v>
       </c>
-      <c r="E18" s="24" t="s">
-        <v>211</v>
-      </c>
-      <c r="F18" s="24" t="s">
+      <c r="E19" s="24" t="s">
         <v>216</v>
       </c>
-      <c r="G18" s="27" t="s">
-        <v>212</v>
-      </c>
-      <c r="H18" s="24" t="s">
-        <v>213</v>
-      </c>
-      <c r="I18" s="28" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
-        <v>207</v>
-      </c>
-      <c r="B19" s="37" t="s">
+      <c r="F19" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="G19" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="H19" s="24" t="s">
         <v>218</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="I19" s="28" t="s">
         <v>219</v>
-      </c>
-      <c r="E19" s="24" t="s">
-        <v>220</v>
-      </c>
-      <c r="F19" s="24" t="s">
-        <v>224</v>
-      </c>
-      <c r="G19" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="H19" s="24" t="s">
-        <v>222</v>
-      </c>
-      <c r="I19" s="28" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="22" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B20" s="37" t="s">
+        <v>232</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>300</v>
+      </c>
+      <c r="D20" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="C20" s="24" t="s">
-        <v>225</v>
-      </c>
-      <c r="D20" s="24" t="s">
-        <v>226</v>
-      </c>
       <c r="E20" s="24" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="H20" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="I20" s="28" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="22" t="s">
         <v>231</v>
       </c>
-      <c r="I20" s="28" t="s">
-        <v>228</v>
+      <c r="B21" s="37" t="s">
+        <v>233</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="D21" s="24" t="s">
+        <v>235</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>234</v>
+      </c>
+      <c r="F21" s="24" t="s">
+        <v>236</v>
+      </c>
+      <c r="G21" s="27" t="s">
+        <v>237</v>
+      </c>
+      <c r="H21" s="24" t="s">
+        <v>238</v>
+      </c>
+      <c r="I21" s="28" t="s">
+        <v>239</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="22"/>
+    <row r="22" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="22" t="s">
+        <v>241</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>252</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>303</v>
+      </c>
+      <c r="D22" s="24" t="s">
+        <v>304</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>309</v>
+      </c>
+      <c r="F22" s="24" t="s">
+        <v>301</v>
+      </c>
+      <c r="G22" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="H22" s="24" t="s">
+        <v>306</v>
+      </c>
+      <c r="I22" s="28" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>253</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>307</v>
+      </c>
+      <c r="D23" s="24" t="s">
+        <v>308</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>314</v>
+      </c>
+      <c r="F23" s="24" t="s">
+        <v>313</v>
+      </c>
+      <c r="G23" s="27" t="s">
+        <v>310</v>
+      </c>
+      <c r="H23" s="24" t="s">
+        <v>312</v>
+      </c>
+      <c r="I23" s="28" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>254</v>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>315</v>
+      </c>
+      <c r="D24" s="24" t="s">
+        <v>320</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>321</v>
+      </c>
+      <c r="F24" s="24" t="s">
+        <v>316</v>
+      </c>
+      <c r="G24" s="27" t="s">
+        <v>317</v>
+      </c>
+      <c r="H24" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="I24" s="28" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" s="44" customFormat="1" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="B25" s="40" t="s">
+        <v>261</v>
+      </c>
+      <c r="C25" s="38" t="s">
+        <v>322</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>325</v>
+      </c>
+      <c r="E25" s="41" t="s">
+        <v>326</v>
+      </c>
+      <c r="F25" s="38" t="s">
+        <v>324</v>
+      </c>
+      <c r="G25" s="42" t="s">
+        <v>323</v>
+      </c>
+      <c r="H25" s="38" t="s">
+        <v>327</v>
+      </c>
+      <c r="I25" s="43" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="22" t="s">
+        <v>245</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>258</v>
+      </c>
+      <c r="C26" s="24" t="s">
+        <v>328</v>
+      </c>
+      <c r="D26" s="24" t="s">
+        <v>329</v>
+      </c>
+      <c r="E26" s="26" t="s">
+        <v>330</v>
+      </c>
+      <c r="F26" s="24" t="s">
+        <v>332</v>
+      </c>
+      <c r="G26" s="27" t="s">
+        <v>333</v>
+      </c>
+      <c r="H26" s="24" t="s">
+        <v>331</v>
+      </c>
+      <c r="I26" s="28" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="22" t="s">
+        <v>246</v>
+      </c>
+      <c r="B27" s="37" t="s">
+        <v>262</v>
+      </c>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="28"/>
+    </row>
+    <row r="28" spans="1:9" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="22" t="s">
+        <v>247</v>
+      </c>
+      <c r="B28" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="28"/>
+    </row>
+    <row r="29" spans="1:9" ht="70" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="22" t="s">
+        <v>248</v>
+      </c>
+      <c r="B29" s="37" t="s">
+        <v>255</v>
+      </c>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="28"/>
+    </row>
+    <row r="30" spans="1:9" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="22" t="s">
+        <v>249</v>
+      </c>
+      <c r="B30" s="37" t="s">
+        <v>257</v>
+      </c>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="28"/>
+    </row>
+    <row r="31" spans="1:9" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="22" t="s">
+        <v>250</v>
+      </c>
+      <c r="B31" s="37" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="28"/>
+    </row>
+    <row r="32" spans="1:9" ht="86" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="B32" s="37" t="s">
+        <v>260</v>
+      </c>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="28"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="30" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0C755C3-D0F0-E142-815A-4D8AA9E2C63B}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" style="10"/>
+    <col min="2" max="2" width="40.83203125" style="2" customWidth="1"/>
+    <col min="3" max="9" width="50.83203125" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="3" customFormat="1" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="20" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="4" customFormat="1" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="B2" s="37" t="s">
+        <v>299</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="14"/>
+    </row>
+    <row r="3" spans="1:9" s="5" customFormat="1" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="B3" s="37" t="s">
+        <v>293</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="14"/>
+    </row>
+    <row r="4" spans="1:9" s="5" customFormat="1" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+    </row>
+    <row r="5" spans="1:9" ht="70" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="14"/>
+    </row>
+    <row r="6" spans="1:9" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="C6" s="24"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="28"/>
+    </row>
+    <row r="7" spans="1:9" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="C7" s="24"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="28"/>
+    </row>
+    <row r="8" spans="1:9" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="C8" s="24"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="28"/>
+    </row>
+    <row r="9" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="B9" s="23"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="28"/>
+    </row>
+    <row r="10" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="B10" s="23"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="26"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="28"/>
+    </row>
+    <row r="11" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
+        <v>272</v>
+      </c>
+      <c r="B11" s="23"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="28"/>
+    </row>
+    <row r="12" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>273</v>
+      </c>
+      <c r="B12" s="37"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="28"/>
+    </row>
+    <row r="13" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="B13" s="37"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="28"/>
+    </row>
+    <row r="14" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="B14" s="37"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="28"/>
+    </row>
+    <row r="15" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>276</v>
+      </c>
+      <c r="B15" s="37"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="28"/>
+    </row>
+    <row r="16" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="B16" s="37"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="28"/>
+    </row>
+    <row r="17" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>278</v>
+      </c>
+      <c r="B17" s="37"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="28"/>
+    </row>
+    <row r="18" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>279</v>
+      </c>
+      <c r="B18" s="23"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="28"/>
+    </row>
+    <row r="19" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="B19" s="37"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="28"/>
+    </row>
+    <row r="20" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="B20" s="37"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="28"/>
+    </row>
+    <row r="21" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
+        <v>282</v>
+      </c>
       <c r="B21" s="37"/>
       <c r="C21" s="24"/>
       <c r="D21" s="24"/>
@@ -6643,6 +8995,137 @@
       <c r="H21" s="24"/>
       <c r="I21" s="28"/>
     </row>
+    <row r="22" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="B22" s="37"/>
+      <c r="C22" s="24"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="28"/>
+    </row>
+    <row r="23" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="B23" s="37"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="26"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="24"/>
+      <c r="I23" s="28"/>
+    </row>
+    <row r="24" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="B24" s="37"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="28"/>
+    </row>
+    <row r="25" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="B25" s="23"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="28"/>
+    </row>
+    <row r="26" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="B26" s="37"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="24"/>
+      <c r="I26" s="28"/>
+    </row>
+    <row r="27" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
+        <v>288</v>
+      </c>
+      <c r="B27" s="37"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="27"/>
+      <c r="H27" s="24"/>
+      <c r="I27" s="28"/>
+    </row>
+    <row r="28" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="B28" s="37"/>
+      <c r="C28" s="24"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="27"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="28"/>
+    </row>
+    <row r="29" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="B29" s="37"/>
+      <c r="C29" s="24"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="27"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="28"/>
+    </row>
+    <row r="30" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="B30" s="37"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="28"/>
+    </row>
+    <row r="31" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="B31" s="37"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="27"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="28"/>
+    </row>
+    <row r="32" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
Deploy: 25 May 2026 · MOTHERHOOD · palette-white · cache vigil-v68
</commit_message>
<xml_diff>
--- a/Vigil_Content_v2.0.xlsx
+++ b/Vigil_Content_v2.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dominicsmacbook/pCloud Drive/Personal/Vigil/Vigil v2/vigil-build/Vigil/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6055D966-6C87-9143-96B1-BD63771C0194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419CC4D7-A394-B042-A420-B60E1FA498FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12000" yWindow="660" windowWidth="17400" windowHeight="18460" activeTab="1" xr2:uid="{D95EB6FA-2870-3442-A079-084F9A0CC5D2}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="26880" windowHeight="18460" activeTab="1" xr2:uid="{D95EB6FA-2870-3442-A079-084F9A0CC5D2}"/>
   </bookViews>
   <sheets>
     <sheet name="April" sheetId="3" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">June!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">May!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="181029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="347">
   <si>
     <t>Hover Links</t>
   </si>
@@ -5607,33 +5607,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">25 May 2026
-Monday
-Ordinary Time · Week One
-Memorial: </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>The Blessed Virgin Mary</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF3D4A5C"/>
-        <rFont val="Georgia"/>
-        <family val="1"/>
-      </rPr>
-      <t>, Mother of the Church</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">30 May 2026
 Saturday
 Ordinary Time · Week One
@@ -5819,12 +5792,6 @@
     <t>04 June 2026
 Thursday
 Ordinary Time · Week Two</t>
-  </si>
-  <si>
-    <t>07 June 2026
-Sunday
-Ordinary Time · Week Three
-Solemnity: The Most Sacred Heart of Jesus</t>
   </si>
   <si>
     <r>
@@ -6820,6 +6787,358 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>CHEERFUL [CHEER-ful]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+The Greek word is </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>hilaros</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (ἱλαρός) — and it is the root of the English word "hilarity." That connection is worth pausing on.
+Hilaros does not mean politely pleasant. It means radiantly, freely glad — the gladness of someone who has nothing left to protect. 
+When </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Paul</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> uses it, as we shall see in today's scripture, he uses it to describe a quality of giving: not the giving of someone discharging an obligation, but of someone who gives because they are genuinely free to.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Philip Neri</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> spent decades in Rome doing exactly that — drawing people to God through prayer, music and long hours of conversation, with a quality of hilaritas that his contemporaries found disarming and, in the best sense, inexplicable. He did not perform joy. He had discovered the freedom that produces it.
+Cheerfulness, in this sense, is not a mood. It is the outward sign of an inward liberty.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">The point is this: the one who sows sparingly will also reap sparingly, and the one who sows bountifully will also reap bountifully. 
+Each of you must give as you have made up your mind, not reluctantly or under compulsion, for God loves a cheerful giver.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+2 Corinthians 9:6–7 — NRSV</t>
+    </r>
+  </si>
+  <si>
+    <t>Lord,
+You love a cheerful giver — not because you need our gifts, but because the freedom to give freely is itself a form of knowing you.
+Where we have given under compulsion — from duty, guilt or the fear of what others will think — forgive us.
+Where we have become calculating with our time, our kindness, our attention: loosen the grip.
+Make us free enough to be generous — not by removing what it costs, but by drawing us close enough to you that the cost no longer has the last word.
+In Christ's name, Amen.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">We are at the start of Ordinary Time, on the Tuesday after Pentecost.
+Today the Church remembers </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Philip Neri,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> a sixteenth-century priest who made holiness so attractive that people came looking for it.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">St Philip Neri (1515–1595 AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Italian priest and founder of the Congregation of the Oratory in Rome. The Church remembers him today; his life gave the word </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>hilaritas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> its most sustained theological expression — a holiness so free and so glad that people came from across the city to be near it.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+St Paul (1st century AD). 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Apostle, missionary and author of letters central to the New Testament. He is featured today because his second letter to the Corinthians gives the day's word its precise scriptural ground: the </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>hilaros</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>-giver is not someone who has mastered generosity, but someone who has been freed from the compulsion not to give.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Most of us know the difference between giving that is free and giving that is not. The free kind — the meal made with genuine pleasure, the time offered without calculating what it costs — feels different to the person receiving it. They can tell. And so can you.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Philip Neri</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> drew people to God not by argument but by the quality of his attention. What they described, centuries later, was something close to delight: the sense that he was genuinely glad they were there.
+There is probably one person in your life it is easy to be generous toward — and one for whom the giving has quietly become a calculation. The difference rarely lies in what they deserve. It usually lies in something in you.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>What has made generosity toward that second person feel like expenditure rather than freedom — and what would change if you brought that tightness to God before you returned to the relationship?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St Philip Neri's</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>cheefulness</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> had a very specific shape: he was never somewhere else. Not managing the conversation, not calculating what the other person was costing him, not half-present while protecting his time. His attention was the form his freedom took.
+Choose one person you will encounter today — in person, by message, or by phone. Decide now to give them your full attention when that moment comes.
+When it arrives, stop composing your reply while they are still speaking or typing. Be entirely there.
+Notice what happens in you as you do it. If it feels like freedom — easy, unguarded, genuinely glad — that is cheefulness. 
+If it feels like effort or cost, that is not a failure. That is the place to pray from: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>Lord, this is where my grip is still tight. Please loosen it. Help me to become your cheerful servant.</t>
+    </r>
+  </si>
+  <si>
+    <t>Red Major</t>
+  </si>
+  <si>
+    <t>White</t>
+  </si>
+  <si>
+    <t>Green</t>
+  </si>
+  <si>
+    <t>07 June 2026
+Sunday
+Ordinary Time · Week Three
+Solemnity: Corpus Christi</t>
+  </si>
+  <si>
+    <t>Palette</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">25 May 2026
+Monday
+Ordinary Time · Week One
+Memorial: The Blessed Virgin Mary, Mother of the Church
+Optional Memorial: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>St. Bede the Venerable</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>, priest and Doctor of the Church</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t xml:space="preserve">Author · Acts of the Apostles (1st century AD). 
 </t>
     </r>
@@ -6831,6 +7150,27 @@
         <family val="1"/>
       </rPr>
       <t>Traditionally identified as Luke, a physician and companion of St Paul, and as the author of both the synonymous Gospel and the Acts of the Apostles. He is featured today because it is in Acts 1 that Mary appears for the last time in the New Testament, as the Church waits for the Spirit that will bring it to life.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Bede the Venerable [c. 673–735]
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF3D4A5C"/>
+        <rFont val="Georgia"/>
+        <family val="1"/>
+      </rPr>
+      <t>An Anglo-Saxon monk, scholar and historian. The Church remembers him as one of the first and greatest interpreters of scripture in the Latin West — a man who spent almost his entire life within a few miles of the Benedictine monastery in Northumbria (northern England) where he was placed as a child.</t>
     </r>
   </si>
 </sst>
@@ -6999,7 +7339,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -7142,11 +7482,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thick">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thick">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thick">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -7279,6 +7658,24 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7596,220 +7993,230 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="10"/>
-    <col min="2" max="2" width="40.83203125" style="2" customWidth="1"/>
-    <col min="3" max="9" width="50.83203125" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="2" max="2" width="40.83203125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" style="2" customWidth="1"/>
+    <col min="4" max="10" width="50.83203125" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="3" customFormat="1" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="45" t="s">
+        <v>344</v>
+      </c>
+      <c r="C1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="D1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="E1" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="F1" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="G1" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="H1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="I1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="J1" s="20" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="4" customFormat="1" ht="291" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="4" customFormat="1" ht="291" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="46"/>
+      <c r="C2" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="H2" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="J2" s="14" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="5" customFormat="1" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" s="5" customFormat="1" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="46"/>
+      <c r="C3" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="F3" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="J3" s="14" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="46"/>
+      <c r="C4" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="E4" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
     </row>
-    <row r="5" spans="1:9" ht="290" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="290" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A5" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="47"/>
+      <c r="C5" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="D5" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="E5" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="F5" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="F5" s="24" t="s">
+      <c r="G5" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="H5" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="I5" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="I5" s="28" t="s">
+      <c r="J5" s="28" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="273" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="273" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="49"/>
+      <c r="C6" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="E6" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="J6" s="15" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="274" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="274" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="50"/>
+      <c r="C7" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="D7" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="D7" s="32" t="s">
+      <c r="E7" s="32" t="s">
         <v>83</v>
       </c>
-      <c r="E7" s="33" t="s">
+      <c r="F7" s="33" t="s">
         <v>84</v>
       </c>
-      <c r="F7" s="31" t="s">
+      <c r="G7" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="G7" s="34" t="s">
+      <c r="H7" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="H7" s="31" t="s">
+      <c r="I7" s="31" t="s">
         <v>87</v>
       </c>
-      <c r="I7" s="35" t="s">
+      <c r="J7" s="35" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="8" spans="1:10" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="31" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" scale="30" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -7818,863 +8225,928 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="10"/>
-    <col min="2" max="2" width="40.83203125" style="2" customWidth="1"/>
-    <col min="3" max="9" width="50.83203125" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="2" max="2" width="40.83203125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" style="2" customWidth="1"/>
+    <col min="4" max="10" width="50.83203125" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="3" customFormat="1" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="45" t="s">
+        <v>344</v>
+      </c>
+      <c r="C1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="D1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="E1" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="F1" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="G1" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="H1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="I1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="J1" s="20" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="4" customFormat="1" ht="274" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="4" customFormat="1" ht="274" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="46"/>
+      <c r="C2" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="H2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="J2" s="14" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:9" s="5" customFormat="1" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" s="5" customFormat="1" ht="257" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="46"/>
+      <c r="C3" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="E3" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="F3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="J3" s="14" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="5" customFormat="1" ht="274" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" s="5" customFormat="1" ht="274" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="46"/>
+      <c r="C4" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I4" s="14" t="s">
+      <c r="J4" s="14" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="291" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="291" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="46"/>
+      <c r="C5" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="H5" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="J5" s="14" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="374" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="374" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="47"/>
+      <c r="C6" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="D6" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="E6" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="F6" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="G6" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="H6" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="I6" s="24" t="s">
         <v>122</v>
       </c>
-      <c r="I6" s="28" t="s">
+      <c r="J6" s="28" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="291" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="291" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="47"/>
+      <c r="C7" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="D7" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="E7" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="F7" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="F7" s="24" t="s">
+      <c r="G7" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="H7" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="I7" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="I7" s="28" t="s">
+      <c r="J7" s="28" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="374" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="374" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="47"/>
+      <c r="C8" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="D8" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="E8" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="F8" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="G8" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="H8" s="27" t="s">
         <v>107</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="I8" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="I8" s="28" t="s">
+      <c r="J8" s="28" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="47"/>
+      <c r="C9" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="D9" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="E9" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="F9" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="F9" s="24" t="s">
+      <c r="G9" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="H9" s="27" t="s">
         <v>129</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="I9" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="I9" s="28" t="s">
+      <c r="J9" s="28" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A10" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="47"/>
+      <c r="C10" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="D10" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="E10" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="F10" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="G10" s="24" t="s">
         <v>136</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="H10" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="I10" s="24" t="s">
         <v>138</v>
       </c>
-      <c r="I10" s="28" t="s">
+      <c r="J10" s="28" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="47"/>
+      <c r="C11" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="D11" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="E11" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="F11" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="F11" s="24" t="s">
+      <c r="G11" s="24" t="s">
         <v>146</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="H11" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="I11" s="24" t="s">
         <v>148</v>
       </c>
-      <c r="I11" s="28" t="s">
+      <c r="J11" s="28" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="B12" s="37" t="s">
+      <c r="B12" s="47"/>
+      <c r="C12" s="37" t="s">
         <v>151</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="D12" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="E12" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="F12" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="F12" s="24" t="s">
+      <c r="G12" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="H12" s="27" t="s">
         <v>158</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="I12" s="24" t="s">
         <v>160</v>
       </c>
-      <c r="I12" s="28" t="s">
+      <c r="J12" s="28" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="B13" s="37" t="s">
+      <c r="B13" s="47"/>
+      <c r="C13" s="37" t="s">
         <v>153</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="D13" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="E13" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="F13" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="F13" s="24" t="s">
+      <c r="G13" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="H13" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="I13" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="I13" s="28" t="s">
+      <c r="J13" s="28" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="B14" s="37" t="s">
+      <c r="B14" s="47"/>
+      <c r="C14" s="37" t="s">
         <v>203</v>
       </c>
-      <c r="C14" s="24" t="s">
+      <c r="D14" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="E14" s="24" t="s">
         <v>225</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="F14" s="26" t="s">
         <v>172</v>
       </c>
-      <c r="F14" s="24" t="s">
+      <c r="G14" s="24" t="s">
         <v>168</v>
       </c>
-      <c r="G14" s="27" t="s">
+      <c r="H14" s="27" t="s">
         <v>169</v>
       </c>
-      <c r="H14" s="24" t="s">
+      <c r="I14" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="I14" s="28" t="s">
+      <c r="J14" s="28" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="22" t="s">
         <v>177</v>
       </c>
-      <c r="B15" s="37" t="s">
+      <c r="B15" s="47"/>
+      <c r="C15" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="D15" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="E15" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="F15" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="F15" s="24" t="s">
+      <c r="G15" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="G15" s="27" t="s">
+      <c r="H15" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="H15" s="24" t="s">
+      <c r="I15" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="I15" s="28" t="s">
+      <c r="J15" s="28" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="22" t="s">
         <v>178</v>
       </c>
-      <c r="B16" s="37" t="s">
+      <c r="B16" s="47"/>
+      <c r="C16" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="D16" s="24" t="s">
         <v>189</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="E16" s="24" t="s">
         <v>190</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="F16" s="26" t="s">
         <v>192</v>
       </c>
-      <c r="F16" s="24" t="s">
+      <c r="G16" s="24" t="s">
         <v>193</v>
       </c>
-      <c r="G16" s="27" t="s">
+      <c r="H16" s="27" t="s">
         <v>194</v>
       </c>
-      <c r="H16" s="24" t="s">
+      <c r="I16" s="24" t="s">
         <v>195</v>
       </c>
-      <c r="I16" s="28" t="s">
+      <c r="J16" s="28" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="374" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="374" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="B17" s="37" t="s">
+      <c r="B17" s="47"/>
+      <c r="C17" s="37" t="s">
         <v>196</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="D17" s="24" t="s">
         <v>197</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="E17" s="24" t="s">
         <v>198</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="F17" s="24" t="s">
         <v>201</v>
       </c>
-      <c r="F17" s="24" t="s">
+      <c r="G17" s="24" t="s">
         <v>202</v>
       </c>
-      <c r="G17" s="27" t="s">
+      <c r="H17" s="27" t="s">
         <v>199</v>
       </c>
-      <c r="H17" s="24" t="s">
+      <c r="I17" s="24" t="s">
         <v>200</v>
       </c>
-      <c r="I17" s="28" t="s">
+      <c r="J17" s="28" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="47"/>
+      <c r="C18" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="D18" s="24" t="s">
         <v>208</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="E18" s="24" t="s">
         <v>212</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="F18" s="24" t="s">
         <v>209</v>
       </c>
-      <c r="F18" s="24" t="s">
+      <c r="G18" s="24" t="s">
         <v>213</v>
       </c>
-      <c r="G18" s="27" t="s">
+      <c r="H18" s="27" t="s">
         <v>210</v>
       </c>
-      <c r="H18" s="24" t="s">
+      <c r="I18" s="24" t="s">
         <v>211</v>
       </c>
-      <c r="I18" s="28" t="s">
+      <c r="J18" s="28" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="390" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="B19" s="37" t="s">
+      <c r="B19" s="47"/>
+      <c r="C19" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="D19" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="E19" s="24" t="s">
         <v>215</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="F19" s="24" t="s">
         <v>216</v>
       </c>
-      <c r="F19" s="24" t="s">
+      <c r="G19" s="24" t="s">
         <v>220</v>
       </c>
-      <c r="G19" s="27" t="s">
+      <c r="H19" s="27" t="s">
         <v>217</v>
       </c>
-      <c r="H19" s="24" t="s">
+      <c r="I19" s="24" t="s">
         <v>218</v>
       </c>
-      <c r="I19" s="28" t="s">
+      <c r="J19" s="28" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="47"/>
+      <c r="C20" s="37" t="s">
         <v>232</v>
       </c>
-      <c r="C20" s="24" t="s">
-        <v>300</v>
-      </c>
       <c r="D20" s="24" t="s">
+        <v>298</v>
+      </c>
+      <c r="E20" s="24" t="s">
         <v>229</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="F20" s="24" t="s">
         <v>221</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="G20" s="24" t="s">
         <v>230</v>
       </c>
-      <c r="G20" s="27" t="s">
+      <c r="H20" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="H20" s="24" t="s">
+      <c r="I20" s="24" t="s">
         <v>224</v>
       </c>
-      <c r="I20" s="28" t="s">
+      <c r="J20" s="28" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
         <v>231</v>
       </c>
-      <c r="B21" s="37" t="s">
+      <c r="B21" s="47"/>
+      <c r="C21" s="37" t="s">
         <v>233</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="D21" s="24" t="s">
         <v>240</v>
       </c>
-      <c r="D21" s="24" t="s">
+      <c r="E21" s="24" t="s">
         <v>235</v>
       </c>
-      <c r="E21" s="26" t="s">
+      <c r="F21" s="26" t="s">
         <v>234</v>
       </c>
-      <c r="F21" s="24" t="s">
+      <c r="G21" s="24" t="s">
         <v>236</v>
       </c>
-      <c r="G21" s="27" t="s">
+      <c r="H21" s="27" t="s">
         <v>237</v>
       </c>
-      <c r="H21" s="24" t="s">
+      <c r="I21" s="24" t="s">
         <v>238</v>
       </c>
-      <c r="I21" s="28" t="s">
+      <c r="J21" s="28" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="22" t="s">
         <v>241</v>
       </c>
-      <c r="B22" s="37" t="s">
+      <c r="B22" s="47"/>
+      <c r="C22" s="37" t="s">
         <v>252</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="D22" s="24" t="s">
+        <v>301</v>
+      </c>
+      <c r="E22" s="24" t="s">
+        <v>302</v>
+      </c>
+      <c r="F22" s="26" t="s">
+        <v>307</v>
+      </c>
+      <c r="G22" s="24" t="s">
+        <v>299</v>
+      </c>
+      <c r="H22" s="27" t="s">
         <v>303</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="I22" s="24" t="s">
         <v>304</v>
       </c>
-      <c r="E22" s="26" t="s">
-        <v>309</v>
-      </c>
-      <c r="F22" s="24" t="s">
-        <v>301</v>
-      </c>
-      <c r="G22" s="27" t="s">
-        <v>305</v>
-      </c>
-      <c r="H22" s="24" t="s">
-        <v>306</v>
-      </c>
-      <c r="I22" s="28" t="s">
-        <v>302</v>
+      <c r="J22" s="28" t="s">
+        <v>300</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="406" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="22" t="s">
         <v>242</v>
       </c>
-      <c r="B23" s="37" t="s">
+      <c r="B23" s="47"/>
+      <c r="C23" s="37" t="s">
         <v>253</v>
       </c>
-      <c r="C23" s="24" t="s">
-        <v>307</v>
-      </c>
       <c r="D23" s="24" t="s">
+        <v>305</v>
+      </c>
+      <c r="E23" s="24" t="s">
+        <v>306</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>312</v>
+      </c>
+      <c r="G23" s="24" t="s">
+        <v>311</v>
+      </c>
+      <c r="H23" s="27" t="s">
         <v>308</v>
       </c>
-      <c r="E23" s="26" t="s">
-        <v>314</v>
-      </c>
-      <c r="F23" s="24" t="s">
-        <v>313</v>
-      </c>
-      <c r="G23" s="27" t="s">
+      <c r="I23" s="24" t="s">
         <v>310</v>
       </c>
-      <c r="H23" s="24" t="s">
-        <v>312</v>
-      </c>
-      <c r="I23" s="28" t="s">
-        <v>311</v>
+      <c r="J23" s="28" t="s">
+        <v>309</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="22" t="s">
         <v>243</v>
       </c>
-      <c r="B24" s="37" t="s">
+      <c r="B24" s="47"/>
+      <c r="C24" s="37" t="s">
         <v>254</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="D24" s="24" t="s">
+        <v>313</v>
+      </c>
+      <c r="E24" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>319</v>
+      </c>
+      <c r="G24" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="H24" s="27" t="s">
         <v>315</v>
       </c>
-      <c r="D24" s="24" t="s">
-        <v>320</v>
-      </c>
-      <c r="E24" s="26" t="s">
-        <v>321</v>
-      </c>
-      <c r="F24" s="24" t="s">
+      <c r="I24" s="24" t="s">
         <v>316</v>
       </c>
-      <c r="G24" s="27" t="s">
+      <c r="J24" s="28" t="s">
         <v>317</v>
       </c>
-      <c r="H24" s="24" t="s">
-        <v>318</v>
-      </c>
-      <c r="I24" s="28" t="s">
-        <v>319</v>
-      </c>
     </row>
-    <row r="25" spans="1:9" s="44" customFormat="1" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" s="44" customFormat="1" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="39" t="s">
         <v>244</v>
       </c>
-      <c r="B25" s="40" t="s">
-        <v>261</v>
-      </c>
-      <c r="C25" s="38" t="s">
+      <c r="B25" s="48" t="s">
+        <v>340</v>
+      </c>
+      <c r="C25" s="40" t="s">
+        <v>260</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>320</v>
+      </c>
+      <c r="E25" s="38" t="s">
+        <v>323</v>
+      </c>
+      <c r="F25" s="41" t="s">
+        <v>324</v>
+      </c>
+      <c r="G25" s="38" t="s">
         <v>322</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="H25" s="42" t="s">
+        <v>321</v>
+      </c>
+      <c r="I25" s="38" t="s">
         <v>325</v>
       </c>
-      <c r="E25" s="41" t="s">
-        <v>326</v>
-      </c>
-      <c r="F25" s="38" t="s">
-        <v>324</v>
-      </c>
-      <c r="G25" s="42" t="s">
-        <v>323</v>
-      </c>
-      <c r="H25" s="38" t="s">
-        <v>327</v>
-      </c>
-      <c r="I25" s="43" t="s">
-        <v>334</v>
+      <c r="J25" s="43" t="s">
+        <v>332</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="22" t="s">
         <v>245</v>
       </c>
-      <c r="B26" s="37" t="s">
-        <v>258</v>
-      </c>
-      <c r="C26" s="24" t="s">
+      <c r="B26" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="C26" s="37" t="s">
+        <v>345</v>
+      </c>
+      <c r="D26" s="24" t="s">
+        <v>326</v>
+      </c>
+      <c r="E26" s="24" t="s">
+        <v>327</v>
+      </c>
+      <c r="F26" s="26" t="s">
         <v>328</v>
       </c>
-      <c r="D26" s="24" t="s">
+      <c r="G26" s="24" t="s">
+        <v>330</v>
+      </c>
+      <c r="H26" s="27" t="s">
+        <v>331</v>
+      </c>
+      <c r="I26" s="24" t="s">
         <v>329</v>
       </c>
-      <c r="E26" s="26" t="s">
-        <v>330</v>
-      </c>
-      <c r="F26" s="24" t="s">
-        <v>332</v>
-      </c>
-      <c r="G26" s="27" t="s">
-        <v>333</v>
-      </c>
-      <c r="H26" s="24" t="s">
-        <v>331</v>
-      </c>
-      <c r="I26" s="28" t="s">
-        <v>335</v>
+      <c r="J26" s="28" t="s">
+        <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="409.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="22" t="s">
         <v>246</v>
       </c>
-      <c r="B27" s="37" t="s">
-        <v>262</v>
-      </c>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="28"/>
+      <c r="B27" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="C27" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="D27" s="24" t="s">
+        <v>336</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>333</v>
+      </c>
+      <c r="F27" s="26" t="s">
+        <v>334</v>
+      </c>
+      <c r="G27" s="24" t="s">
+        <v>338</v>
+      </c>
+      <c r="H27" s="27" t="s">
+        <v>335</v>
+      </c>
+      <c r="I27" s="24" t="s">
+        <v>339</v>
+      </c>
+      <c r="J27" s="28" t="s">
+        <v>337</v>
+      </c>
     </row>
-    <row r="28" spans="1:9" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="22" t="s">
         <v>247</v>
       </c>
-      <c r="B28" s="37" t="s">
+      <c r="B28" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="C28" s="37" t="s">
         <v>256</v>
       </c>
-      <c r="C28" s="24"/>
       <c r="D28" s="24"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="28"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="28"/>
     </row>
-    <row r="29" spans="1:9" ht="70" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="70" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A29" s="22" t="s">
         <v>248</v>
       </c>
-      <c r="B29" s="37" t="s">
+      <c r="B29" s="47" t="s">
+        <v>342</v>
+      </c>
+      <c r="C29" s="37" t="s">
         <v>255</v>
       </c>
-      <c r="C29" s="24"/>
       <c r="D29" s="24"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="28"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="24"/>
+      <c r="J29" s="28"/>
     </row>
-    <row r="30" spans="1:9" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A30" s="22" t="s">
         <v>249</v>
       </c>
-      <c r="B30" s="37" t="s">
+      <c r="B30" s="47" t="s">
+        <v>342</v>
+      </c>
+      <c r="C30" s="37" t="s">
         <v>257</v>
       </c>
-      <c r="C30" s="24"/>
       <c r="D30" s="24"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="28"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="28"/>
     </row>
-    <row r="31" spans="1:9" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A31" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="B31" s="37" t="s">
-        <v>259</v>
-      </c>
-      <c r="C31" s="24"/>
+      <c r="B31" s="47" t="s">
+        <v>342</v>
+      </c>
+      <c r="C31" s="37" t="s">
+        <v>258</v>
+      </c>
       <c r="D31" s="24"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="24"/>
-      <c r="I31" s="28"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="28"/>
     </row>
-    <row r="32" spans="1:9" ht="86" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="86" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A32" s="22" t="s">
         <v>251</v>
       </c>
-      <c r="B32" s="37" t="s">
-        <v>260</v>
-      </c>
-      <c r="C32" s="24"/>
+      <c r="B32" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="C32" s="37" t="s">
+        <v>259</v>
+      </c>
       <c r="D32" s="24"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="28"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="27"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="28"/>
     </row>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="30" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" scale="27" fitToHeight="8" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -8683,452 +9155,546 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="10"/>
-    <col min="2" max="2" width="40.83203125" style="2" customWidth="1"/>
-    <col min="3" max="9" width="50.83203125" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="2" max="2" width="40.83203125" style="10" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" style="2" customWidth="1"/>
+    <col min="4" max="10" width="50.83203125" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="3" customFormat="1" ht="19" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="45" t="s">
+        <v>344</v>
+      </c>
+      <c r="C1" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="D1" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="E1" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="F1" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="G1" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="H1" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="I1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="J1" s="20" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="4" customFormat="1" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="4" customFormat="1" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="C2" s="37" t="s">
+        <v>297</v>
+      </c>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="14"/>
+    </row>
+    <row r="3" spans="1:10" s="5" customFormat="1" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="B2" s="37" t="s">
-        <v>299</v>
-      </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="14"/>
+      <c r="B3" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C3" s="37" t="s">
+        <v>292</v>
+      </c>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="14"/>
     </row>
-    <row r="3" spans="1:9" s="5" customFormat="1" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+    <row r="4" spans="1:10" s="5" customFormat="1" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="B4" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="14"/>
+    </row>
+    <row r="5" spans="1:10" ht="70" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="14"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="14"/>
     </row>
-    <row r="4" spans="1:9" s="5" customFormat="1" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="B4" s="6" t="s">
+    <row r="6" spans="1:10" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="D6" s="24"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="28"/>
+    </row>
+    <row r="7" spans="1:10" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="14"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="28"/>
     </row>
-    <row r="5" spans="1:9" ht="70" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
-        <v>266</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="14"/>
+    <row r="8" spans="1:10" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>268</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>343</v>
+      </c>
+      <c r="D8" s="24"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="28"/>
     </row>
-    <row r="6" spans="1:9" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="28"/>
+    <row r="9" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C9" s="23"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="28"/>
     </row>
-    <row r="7" spans="1:9" ht="104" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="28"/>
+    <row r="10" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C10" s="23"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="28"/>
     </row>
-    <row r="8" spans="1:9" ht="87" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>269</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>295</v>
-      </c>
-      <c r="C8" s="24"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="28"/>
+    <row r="11" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C11" s="23"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="28"/>
     </row>
-    <row r="9" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
-        <v>270</v>
-      </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="28"/>
+    <row r="12" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>272</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="C12" s="37"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="28"/>
     </row>
-    <row r="10" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="28"/>
+    <row r="13" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>273</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C13" s="37"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="28"/>
     </row>
-    <row r="11" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
-        <v>272</v>
-      </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="28"/>
+    <row r="14" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C14" s="37"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="28"/>
     </row>
-    <row r="12" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="B12" s="37"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="28"/>
+    <row r="15" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C15" s="37"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="28"/>
     </row>
-    <row r="13" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
-        <v>274</v>
-      </c>
-      <c r="B13" s="37"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="28"/>
+    <row r="16" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>276</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C16" s="37"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="28"/>
     </row>
-    <row r="14" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
-        <v>275</v>
-      </c>
-      <c r="B14" s="37"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="28"/>
-    </row>
-    <row r="15" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
-        <v>276</v>
-      </c>
-      <c r="B15" s="37"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="28"/>
-    </row>
-    <row r="16" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+    <row r="17" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
         <v>277</v>
       </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="28"/>
-    </row>
-    <row r="17" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
-        <v>278</v>
-      </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="24"/>
+      <c r="B17" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C17" s="37"/>
       <c r="D17" s="24"/>
       <c r="E17" s="24"/>
       <c r="F17" s="24"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="28"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="28"/>
     </row>
-    <row r="18" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>279</v>
-      </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="24"/>
+        <v>278</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C18" s="23"/>
       <c r="D18" s="24"/>
       <c r="E18" s="24"/>
       <c r="F18" s="24"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="28"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="28"/>
     </row>
-    <row r="19" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>280</v>
-      </c>
-      <c r="B19" s="37"/>
-      <c r="C19" s="24"/>
+        <v>279</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C19" s="37"/>
       <c r="D19" s="24"/>
       <c r="E19" s="24"/>
       <c r="F19" s="24"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="28"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="28"/>
     </row>
-    <row r="20" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>281</v>
-      </c>
-      <c r="B20" s="37"/>
-      <c r="C20" s="24"/>
+        <v>280</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C20" s="37"/>
       <c r="D20" s="24"/>
       <c r="E20" s="24"/>
       <c r="F20" s="24"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="28"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="28"/>
     </row>
-    <row r="21" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C21" s="37"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="28"/>
+    </row>
+    <row r="22" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
         <v>282</v>
       </c>
-      <c r="B21" s="37"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="26"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="28"/>
+      <c r="B22" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C22" s="37"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="28"/>
     </row>
-    <row r="22" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+    <row r="23" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
         <v>283</v>
       </c>
-      <c r="B22" s="37"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="28"/>
+      <c r="B23" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="C23" s="37"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="26"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="24"/>
+      <c r="J23" s="28"/>
     </row>
-    <row r="23" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+    <row r="24" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
         <v>284</v>
       </c>
-      <c r="B23" s="37"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="26"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="28"/>
+      <c r="B24" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C24" s="37"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="26"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="28"/>
     </row>
-    <row r="24" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+    <row r="25" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
         <v>285</v>
       </c>
-      <c r="B24" s="37"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="28"/>
+      <c r="B25" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C25" s="23"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="26"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="28"/>
     </row>
-    <row r="25" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+    <row r="26" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="28"/>
+      <c r="B26" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C26" s="37"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="24"/>
+      <c r="J26" s="28"/>
     </row>
-    <row r="26" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+    <row r="27" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="B26" s="37"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="26"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="28"/>
+      <c r="B27" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="C27" s="37"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="27"/>
+      <c r="I27" s="24"/>
+      <c r="J27" s="28"/>
     </row>
-    <row r="27" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+    <row r="28" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
         <v>288</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="28"/>
+      <c r="B28" s="13" t="s">
+        <v>341</v>
+      </c>
+      <c r="C28" s="37"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="26"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="27"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="28"/>
     </row>
-    <row r="28" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+    <row r="29" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
         <v>289</v>
       </c>
-      <c r="B28" s="37"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="28"/>
+      <c r="B29" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="C29" s="37"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="27"/>
+      <c r="I29" s="24"/>
+      <c r="J29" s="28"/>
     </row>
-    <row r="29" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+    <row r="30" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
         <v>290</v>
       </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="28"/>
+      <c r="B30" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="C30" s="37"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="28"/>
     </row>
-    <row r="30" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
+    <row r="31" spans="1:10" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
         <v>291</v>
       </c>
-      <c r="B30" s="37"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="28"/>
+      <c r="B31" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="C31" s="37"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="27"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="28"/>
     </row>
-    <row r="31" spans="1:9" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
-        <v>292</v>
-      </c>
-      <c r="B31" s="37"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="24"/>
-      <c r="I31" s="28"/>
-    </row>
-    <row r="32" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:10" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="30" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" scale="27" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>